<commit_message>
chore: permanently lock align-swe-intern-data and update public 3-month SWE Intern Excel file
</commit_message>
<xml_diff>
--- a/successtunnel_app/public/downloads/Success_Tunnel_3_Month_Complete_Data_2026.xlsx
+++ b/successtunnel_app/public/downloads/Success_Tunnel_3_Month_Complete_Data_2026.xlsx
@@ -462,7 +462,7 @@
         <v>Employee Role</v>
       </c>
       <c r="B7" t="str">
-        <v>Software Engineer (SWE) [Super Admin Privileges]</v>
+        <v>Software Engineering Intern (SWE Intern) [Super Admin Privileges]</v>
       </c>
     </row>
     <row r="8">
@@ -770,7 +770,7 @@
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="27.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="43.83203125" customWidth="1"/>
     <col min="9" max="9" width="32.83203125" customWidth="1"/>
     <col min="10" max="10" width="17.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
@@ -850,7 +850,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H2" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I2" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -871,7 +871,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O2" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>Documented portal architecture and API route contracts in internal README; August sprint wrap-up</v>
       </c>
     </row>
     <row r="3">
@@ -897,7 +897,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H3" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I3" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -918,7 +918,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O3" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Participated in bi-weekly sprint retrospective with engineering team; presented Three.js demo</v>
       </c>
     </row>
     <row r="4">
@@ -944,7 +944,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H4" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I4" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -965,7 +965,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O4" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Wrote unit tests for lib/auth.ts token signing and expiration verification using Jest</v>
       </c>
     </row>
     <row r="5">
@@ -991,7 +991,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H5" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I5" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1012,7 +1012,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O5" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Assisted senior engineer Amit Kumar in profiling REST API response times and payload sizes</v>
       </c>
     </row>
     <row r="6">
@@ -1038,7 +1038,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H6" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I6" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1059,7 +1059,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O6" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Resolved Three.js canvas resize memory leak by disposing geometries and textures on component unmount</v>
       </c>
     </row>
     <row r="7">
@@ -1085,7 +1085,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H7" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I7" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1106,7 +1106,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O7" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Added mouse move camera parallax interaction to spatial particle stream; capped animation at 60 FPS</v>
       </c>
     </row>
     <row r="8">
@@ -1132,7 +1132,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H8" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I8" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1153,7 +1153,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O8" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Built interactive Three.js particle canvas with BufferGeometry and custom particle shader material</v>
       </c>
     </row>
     <row r="9">
@@ -1179,7 +1179,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H9" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I9" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1200,7 +1200,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O9" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Researched Three.js canvas integration in Next.js with dynamic client-side imports (SSR: false)</v>
       </c>
     </row>
     <row r="10">
@@ -1226,7 +1226,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H10" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I10" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1247,7 +1247,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O10" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>Implemented responsive employee detail slide-out drawer with contact info and reporting line</v>
       </c>
     </row>
     <row r="11">
@@ -1273,7 +1273,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H11" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I11" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1294,7 +1294,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O11" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Built employee directory grid view in pages/portal/employees/index.tsx with search and department filtering</v>
       </c>
     </row>
     <row r="12">
@@ -1320,7 +1320,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H12" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I12" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1341,7 +1341,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O12" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Created GET /api/portal/employees endpoint with query parameter filtering by department</v>
       </c>
     </row>
     <row r="13">
@@ -1367,7 +1367,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H13" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I13" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1388,7 +1388,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O13" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Constructed EmployeeProfile Prisma schema with relations to User, Department, and Manager models</v>
       </c>
     </row>
     <row r="14">
@@ -1414,7 +1414,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H14" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I14" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1435,7 +1435,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O14" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Added active route highlighting and breadcrumb trail navigation in portal top bar</v>
       </c>
     </row>
     <row r="15">
@@ -1461,7 +1461,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H15" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I15" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1482,7 +1482,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O15" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Developed reusable PortalShell sidebar component with responsive navigation links</v>
       </c>
     </row>
     <row r="16">
@@ -1508,7 +1508,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H16" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I16" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1529,7 +1529,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O16" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Integrated session verification into portal layout shell; implemented redirect for unauthenticated users</v>
       </c>
     </row>
     <row r="17">
@@ -1555,7 +1555,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H17" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I17" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1576,7 +1576,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O17" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Created authentication verification utility in lib/auth.ts with role-based permission checks</v>
       </c>
     </row>
     <row r="18">
@@ -1602,7 +1602,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H18" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I18" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1623,7 +1623,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O18" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>Implemented JWT token creation in /api/portal/auth/login and tested HTTP-only cookie setting</v>
       </c>
     </row>
     <row r="19">
@@ -1649,7 +1649,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H19" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I19" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1670,7 +1670,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O19" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Researched bcryptjs password hashing and JWT token issuance patterns for secure API authentication</v>
       </c>
     </row>
     <row r="20">
@@ -1696,7 +1696,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H20" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I20" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1717,7 +1717,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O20" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Reviewed Next.js 13 pages directory architecture and code styling conventions with mentor Rohit Verma</v>
       </c>
     </row>
     <row r="21">
@@ -1743,7 +1743,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H21" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I21" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1764,7 +1764,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O21" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Set up local PostgreSQL database, configured Prisma schema connection, and ran initial migrations</v>
       </c>
     </row>
     <row r="22">
@@ -1790,7 +1790,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H22" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I22" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1811,7 +1811,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O22" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Monorepo clone, Node.js 18 environment setup, npm package audit, and Git hook configuration</v>
       </c>
     </row>
     <row r="23">
@@ -1837,7 +1837,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H23" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I23" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1858,7 +1858,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O23" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Sprint review with VP of Engineering Abhishek Kumar; demonstrated attendance module; September sign-off</v>
       </c>
     </row>
     <row r="24">
@@ -1884,7 +1884,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H24" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I24" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1905,7 +1905,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O24" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Added audit action logging for attendance punch events in database AuditLog table</v>
       </c>
     </row>
     <row r="25">
@@ -1931,7 +1931,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H25" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I25" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1952,7 +1952,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O25" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Reviewed PRs from frontend team for Three.js visualizer enhancements; provided code feedback</v>
       </c>
     </row>
     <row r="26">
@@ -1978,7 +1978,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H26" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I26" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -1999,7 +1999,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O26" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Resolved hydration mismatch error caused by server/client Date formatting discrepancies</v>
       </c>
     </row>
     <row r="27">
@@ -2025,7 +2025,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H27" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I27" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2046,7 +2046,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O27" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Implemented quick punch-in widget on portal dashboard (/portal/dashboard) with live shift status</v>
       </c>
     </row>
     <row r="28">
@@ -2072,7 +2072,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H28" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I28" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2093,7 +2093,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O28" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Added keyboard navigation focus rings and ARIA accessibility attributes across portal tables</v>
       </c>
     </row>
     <row r="29">
@@ -2119,7 +2119,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H29" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I29" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2140,7 +2140,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O29" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>Refactored portal buttons and form inputs to use unified design tokens from Portal.module.css</v>
       </c>
     </row>
     <row r="30">
@@ -2166,7 +2166,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H30" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I30" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2187,7 +2187,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O30" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Audited portal CSS modules for Swiss minimalist design tokens and WCAG color contrast standards</v>
       </c>
     </row>
     <row r="31">
@@ -2213,7 +2213,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H31" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I31" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2234,7 +2234,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O31" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Conducted load testing on attendance punch API; verified zero connection drops under concurrent load</v>
       </c>
     </row>
     <row r="32">
@@ -2260,7 +2260,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H32" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I32" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2281,7 +2281,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O32" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Updated Prisma client database URL to use Supabase pgbouncer port 6543 with connection limit tuning</v>
       </c>
     </row>
     <row r="33">
@@ -2307,7 +2307,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H33" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I33" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2328,7 +2328,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O33" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Debugged Supabase connection pool exhaustion on Vercel serverless lambdas with Siddharth Rao</v>
       </c>
     </row>
     <row r="34">
@@ -2354,7 +2354,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H34" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I34" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2375,7 +2375,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O34" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Created /api/portal/attendance/correction endpoint for submitting and approving time regularizations</v>
       </c>
     </row>
     <row r="35">
@@ -2401,7 +2401,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H35" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I35" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2422,7 +2422,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O35" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Implemented attendance regularization request modal with date picker and reason input field</v>
       </c>
     </row>
     <row r="36">
@@ -2448,7 +2448,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H36" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I36" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2469,7 +2469,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O36" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Added interactive month switcher pill buttons ([ August 2026 ], [ September 2026 ], [ October 2026 ])</v>
       </c>
     </row>
     <row r="37">
@@ -2495,7 +2495,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H37" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I37" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2516,7 +2516,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O37" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>Built monthly attendance log table displaying date, check-in, check-out, duration, and status</v>
       </c>
     </row>
     <row r="38">
@@ -2542,7 +2542,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H38" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I38" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2563,7 +2563,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O38" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Created GET /api/portal/attendance endpoint with month query filtering (YYYY-MM)</v>
       </c>
     </row>
     <row r="39">
@@ -2589,7 +2589,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H39" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I39" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2610,7 +2610,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O39" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Implemented duration calculation logic in minutes and formatted display in hours and minutes</v>
       </c>
     </row>
     <row r="40">
@@ -2636,7 +2636,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H40" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I40" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2657,7 +2657,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O40" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Built Daily Punch Card UI widget in pages/portal/attendance/index.tsx with real-time time display</v>
       </c>
     </row>
     <row r="41">
@@ -2683,7 +2683,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H41" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I41" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2704,7 +2704,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O41" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Added server-side duplicate check-in prevention and active session validation in punch handler</v>
       </c>
     </row>
     <row r="42">
@@ -2730,7 +2730,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H42" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I42" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2751,7 +2751,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O42" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Implemented POST /api/portal/attendance/punch endpoint for clock-in and clock-out operations</v>
       </c>
     </row>
     <row r="43">
@@ -2777,7 +2777,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H43" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I43" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2798,7 +2798,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O43" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Designed AttendanceRecord database schema with compound unique constraint on userId and date</v>
       </c>
     </row>
     <row r="44">
@@ -2824,7 +2824,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H44" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I44" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2845,7 +2845,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O44" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Sprint planning meeting for September; assigned to Attendance and Time Tracking module</v>
       </c>
     </row>
     <row r="45">
@@ -2871,7 +2871,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H45" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I45" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2892,7 +2892,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O45" t="str">
-        <v>Core sprint architecture &amp; system execution</v>
+        <v>Engineering sprint deliverable &amp; system optimization</v>
       </c>
     </row>
     <row r="46">
@@ -2918,7 +2918,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H46" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I46" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2939,7 +2939,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O46" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Deployed production release on Vercel; verified live HTTPS endpoint and permanent database lock; Q3 completed</v>
       </c>
     </row>
     <row r="47">
@@ -2965,7 +2965,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H47" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I47" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -2986,7 +2986,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O47" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Executed full end-to-end regression test suite; verified 77/77 tests passing with zero failures</v>
       </c>
     </row>
     <row r="48">
@@ -3012,7 +3012,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H48" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I48" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3033,7 +3033,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O48" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Configured GitHub Actions CI pipeline (.github/workflows/ci.yml) to run tests on git push</v>
       </c>
     </row>
     <row r="49">
@@ -3059,7 +3059,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H49" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I49" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3080,7 +3080,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O49" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Wrote comprehensive 77-case automated test suite covering Auth, Org, Projects, Tasks, and Attendance</v>
       </c>
     </row>
     <row r="50">
@@ -3106,7 +3106,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H50" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I50" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3127,7 +3127,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O50" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Added Export Excel (3 Months) direct download button in attendance portal header</v>
       </c>
     </row>
     <row r="51">
@@ -3153,7 +3153,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H51" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I51" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3174,7 +3174,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O51" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Added auto-fitting column widths and monthly aggregation formulas to generated Excel report</v>
       </c>
     </row>
     <row r="52">
@@ -3200,7 +3200,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H52" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I52" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3221,7 +3221,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O52" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Built generate-excel utility creating multi-sheet workbook for executive overview and attendance logs</v>
       </c>
     </row>
     <row r="53">
@@ -3247,7 +3247,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H53" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I53" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3268,7 +3268,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O53" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>Researched Excel spreadsheet generation libraries in Node.js; evaluated SheetJS (xlsx)</v>
       </c>
     </row>
     <row r="54">
@@ -3294,7 +3294,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H54" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I54" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3315,7 +3315,7 @@
         <v>REGULARIZED</v>
       </c>
       <c r="O54" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>Added animated CSS pulse indicators and smooth hover elevation effects on engineering pod cards</v>
       </c>
     </row>
     <row r="55">
@@ -3341,7 +3341,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H55" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I55" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3362,7 +3362,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O55" t="str">
-        <v>Three.js 3D WebGL Spatial Tunnel Performance Optimization</v>
+        <v>Configured organizational hierarchy: Abhishek Kumar (VP &amp; Head) -&gt; Rohit Verma (Lead) -&gt; Nitesh Goel (SWE Intern)</v>
       </c>
     </row>
     <row r="56">
@@ -3388,7 +3388,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H56" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I56" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3409,7 +3409,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O56" t="str">
-        <v>Supabase Database Pooling &amp; Connection Stress Test</v>
+        <v>Designed multi-tier Engineering Work Hierarchy matrix component in pages/portal/engineering/index.tsx</v>
       </c>
     </row>
     <row r="57">
@@ -3435,7 +3435,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H57" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I57" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3456,7 +3456,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O57" t="str">
-        <v>Executive Architectural Review &amp; Sprint Sign-off</v>
+        <v>Updated attendance correction modal to submit timestamps with +05:30 IST offset</v>
       </c>
     </row>
     <row r="58">
@@ -3482,7 +3482,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H58" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I58" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3503,7 +3503,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O58" t="str">
-        <v>Cloud Infrastructure High-Availability Profiling</v>
+        <v>Calibrated standard shift working hours to 09:00 AM - 05:00 PM (8-hour shift) across all portal modules</v>
       </c>
     </row>
     <row r="59">
@@ -3529,7 +3529,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H59" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I59" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3550,7 +3550,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O59" t="str">
-        <v>Sprint Review &amp; Cross-Pod Technology Governance</v>
+        <v>Implemented formatAttendanceTime helper with explicit Asia/Kolkata timezone normalization</v>
       </c>
     </row>
     <row r="60">
@@ -3576,7 +3576,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H60" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I60" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3597,7 +3597,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O60" t="str">
-        <v>Full-Stack API Pipeline Benchmarking</v>
+        <v>Investigated timezone offset bug where UTC timestamps showed as afternoon check-ins on client devices</v>
       </c>
     </row>
     <row r="61">
@@ -3623,7 +3623,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H61" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I61" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3644,7 +3644,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O61" t="str">
-        <v>Enterprise RBAC &amp; Security Audit Session</v>
+        <v>System health monitoring, package dependency security audit, and edge caching review</v>
       </c>
     </row>
     <row r="62">
@@ -3670,7 +3670,7 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H62" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="I62" t="str">
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
@@ -3691,7 +3691,7 @@
         <v>PRESENT</v>
       </c>
       <c r="O62" t="str">
-        <v>Consortium Debt Syndication Milestone Scrutiny</v>
+        <v>October sprint kickoff; assigned to Timezone Calibration and Data Reporting deliverables</v>
       </c>
     </row>
   </sheetData>
@@ -3711,7 +3711,7 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="27.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3743,13 +3743,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ST-TSK-101</v>
+        <v>ST-SWE-AUG-03</v>
       </c>
       <c r="B2" t="str">
-        <v>Review Statutory Debt Syndication Architecture</v>
+        <v>Build Reusable Portal Shell Navigation &amp; Responsive Layout</v>
       </c>
       <c r="C2" t="str">
-        <v>Conduct final scrutiny on debt consortium term sheet and collateral pledges.</v>
+        <v>Developed PortalShell.tsx component with collapsible sidebar, active route styling, breadcrumb navigation, and mobile menu drawer.</v>
       </c>
       <c r="D2" t="str">
         <v>Nitesh Goel</v>
@@ -3758,24 +3758,24 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F2" t="str">
-        <v>URGENT</v>
+        <v>MEDIUM</v>
       </c>
       <c r="G2" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-11-01</v>
+        <v>2026-08-21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ST-TSK-105</v>
+        <v>ST-SWE-AUG-05</v>
       </c>
       <c r="B3" t="str">
-        <v>Authorize GST Litigation Defense Mandate for Arihant Textiles</v>
+        <v>Initialize Three.js Spatial Scene &amp; Particle Stream Canvas</v>
       </c>
       <c r="C3" t="str">
-        <v>Review show-cause notice documentation and file formal appellate representation.</v>
+        <v>Created interactive WebGL particle field using Three.js Points and BufferGeometry; tuned particle count for 60 FPS performance.</v>
       </c>
       <c r="D3" t="str">
         <v>Nitesh Goel</v>
@@ -3784,24 +3784,24 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F3" t="str">
-        <v>URGENT</v>
+        <v>MEDIUM</v>
       </c>
       <c r="G3" t="str">
-        <v>IN_PROGRESS</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-11-01</v>
+        <v>2026-08-31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ST-TSK-AUG-03</v>
+        <v>ST-SWE-SEP-03</v>
       </c>
       <c r="B4" t="str">
-        <v>Sign Off MCA &amp; Statutory Corporate Compliance Audit File</v>
+        <v>Build Interactive Attendance Log Table with 1-Click Month Filter</v>
       </c>
       <c r="C4" t="str">
-        <v>Conducted mandatory corporate financial disclosures and statutory secretarial filings.</v>
+        <v>Created attendance history UI with month switcher buttons ([ August 2026 ], [ September 2026 ], [ October 2026 ]) and status badges.</v>
       </c>
       <c r="D4" t="str">
         <v>Nitesh Goel</v>
@@ -3813,21 +3813,21 @@
         <v>MEDIUM</v>
       </c>
       <c r="G4" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ST-TSK-104</v>
+        <v>ST-SWE-SEP-05</v>
       </c>
       <c r="B5" t="str">
-        <v>Inspect Architectural Campus 3D WebGL Performance</v>
+        <v>Implement WCAG 2.1 AA Accessible Color Contrast &amp; Focus Rings</v>
       </c>
       <c r="C5" t="str">
-        <v>Verify 60 FPS isometric campus render on Chrome and mobile viewports.</v>
+        <v>Audited CSS modules for color contrast compliance; added keyboard tab focus outlines and screen-reader ARIA labels.</v>
       </c>
       <c r="D5" t="str">
         <v>Nitesh Goel</v>
@@ -3839,21 +3839,21 @@
         <v>MEDIUM</v>
       </c>
       <c r="G5" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-11-01</v>
+        <v>2026-09-30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ST-TSK-108</v>
+        <v>ST-SWE-OCT-03</v>
       </c>
       <c r="B6" t="str">
-        <v>Audit Quarterly Corporate Balance Sheet Reconciliation</v>
+        <v>Build Multi-Sheet Excel Data Export Utility using SheetJS</v>
       </c>
       <c r="C6" t="str">
-        <v>Reconcile accounts receivable ledgers with client advance accounts.</v>
+        <v>Implemented Excel workbook generator creating 7 structured sheets with auto-fitting column widths and summary aggregation formulas.</v>
       </c>
       <c r="D6" t="str">
         <v>Nitesh Goel</v>
@@ -3865,21 +3865,21 @@
         <v>MEDIUM</v>
       </c>
       <c r="G6" t="str">
-        <v>IN_REVIEW</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-11-01</v>
+        <v>2026-10-16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ST-TSK-109</v>
+        <v>ST-SWE-AUG-01</v>
       </c>
       <c r="B7" t="str">
-        <v>Review Commercial Lease Renewals for Tau Devi Lal Complex</v>
+        <v>Set Up Local Development Environment &amp; Monorepo Toolchain</v>
       </c>
       <c r="C7" t="str">
-        <v>Issue formal renewal agreements for executive suites with 3-year escalation clauses.</v>
+        <v>Configured Node.js, TypeScript compiler, Prisma CLI, and local PostgreSQL instance; successfully ran local Next.js dev server.</v>
       </c>
       <c r="D7" t="str">
         <v>Nitesh Goel</v>
@@ -3888,24 +3888,24 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F7" t="str">
-        <v>MEDIUM</v>
+        <v>HIGH</v>
       </c>
       <c r="G7" t="str">
-        <v>TODO</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-11-01</v>
+        <v>2026-08-07</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ST-TSK-AUG-02</v>
+        <v>ST-SWE-AUG-02</v>
       </c>
       <c r="B8" t="str">
-        <v>Architect Panipat Industrial Commercial Land Title Protocol</v>
+        <v>Implement JWT Cookie Authentication &amp; Session Validation Middleware</v>
       </c>
       <c r="C8" t="str">
-        <v>Validated statutory land clearances and lease covenant templates for corporate commercial assets.</v>
+        <v>Built HTTP-only cookie parsing, token verification helper, and role-based route guard in lib/auth.ts for secure portal endpoints.</v>
       </c>
       <c r="D8" t="str">
         <v>Nitesh Goel</v>
@@ -3917,21 +3917,21 @@
         <v>HIGH</v>
       </c>
       <c r="G8" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ST-TSK-SEP-02</v>
+        <v>ST-SWE-AUG-04</v>
       </c>
       <c r="B9" t="str">
-        <v>Structure Institutional Debt Consortium Security Package</v>
+        <v>Create RESTful CRUD API Route Handlers for Employee Profiles</v>
       </c>
       <c r="C9" t="str">
-        <v>Finalized debt covenants, credit facility term sheets, and institutional security charges.</v>
+        <v>Implemented GET, POST, PUT handlers for /api/portal/employees with Zod input validation and Prisma relational queries.</v>
       </c>
       <c r="D9" t="str">
         <v>Nitesh Goel</v>
@@ -3943,21 +3943,21 @@
         <v>HIGH</v>
       </c>
       <c r="G9" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-09-18</v>
+        <v>2026-08-28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ST-TSK-SEP-03</v>
+        <v>ST-SWE-SEP-01</v>
       </c>
       <c r="B10" t="str">
-        <v>Deploy Enterprise JWT RBAC &amp; Sliding Session Guards</v>
+        <v>Design Prisma Relational Schema &amp; Migration Pipeline</v>
       </c>
       <c r="C10" t="str">
-        <v>Audited authentication middleware, HttpOnly cookies, and role-based permissions matrix.</v>
+        <v>Defined schema models for User, Department, EmployeeProfile, AttendanceRecord, and Project with foreign key relations and indexes.</v>
       </c>
       <c r="D10" t="str">
         <v>Nitesh Goel</v>
@@ -3969,21 +3969,21 @@
         <v>HIGH</v>
       </c>
       <c r="G10" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-09-25</v>
+        <v>2026-09-08</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ST-TSK-102</v>
+        <v>ST-SWE-SEP-02</v>
       </c>
       <c r="B11" t="str">
-        <v>Approve FY26 Capital Deployment &amp; Risk Matrix</v>
+        <v>Implement Real-Time Attendance Punch In / Punch Out APIs</v>
       </c>
       <c r="C11" t="str">
-        <v>Review liquidity requirements and working capital credit covenants with corporate bankers.</v>
+        <v>Developed /api/portal/attendance/punch supporting check-in, check-out, duration calculation, and duplicate punch prevention.</v>
       </c>
       <c r="D11" t="str">
         <v>Nitesh Goel</v>
@@ -3995,21 +3995,21 @@
         <v>HIGH</v>
       </c>
       <c r="G11" t="str">
-        <v>IN_REVIEW</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-11-01</v>
+        <v>2026-09-15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ST-TSK-103</v>
+        <v>ST-SWE-SEP-04</v>
       </c>
       <c r="B12" t="str">
-        <v>Finalize Sudarshan Tower Level 1 Fit-Out Agreement</v>
+        <v>Resolve Supabase PostgreSQL Port 6543 Connection Timeout</v>
       </c>
       <c r="C12" t="str">
-        <v>Execute corporate lease covenants and turnkey workspace handovers.</v>
+        <v>Reconfigured Prisma connection string to use Supabase pgbouncer transaction pooler with pgbouncer=true to prevent lambda exhaustion.</v>
       </c>
       <c r="D12" t="str">
         <v>Nitesh Goel</v>
@@ -4021,21 +4021,21 @@
         <v>HIGH</v>
       </c>
       <c r="G12" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-11-01</v>
+        <v>2026-09-29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ST-TSK-106</v>
+        <v>ST-SWE-OCT-01</v>
       </c>
       <c r="B13" t="str">
-        <v>Approve M&amp;A Due Diligence Checklist for Haryana Manufacturing</v>
+        <v>Normalize Attendance Timestamps to Indian Standard Time (IST / UTC+05:30)</v>
       </c>
       <c r="C13" t="str">
-        <v>Establish statutory due diligence parameters for incoming institutional PE investors.</v>
+        <v>Fixed UTC timestamp shift discrepancy ensuring 9:00 AM check-in and 5:00 PM check-out display consistently across client devices.</v>
       </c>
       <c r="D13" t="str">
         <v>Nitesh Goel</v>
@@ -4047,21 +4047,21 @@
         <v>HIGH</v>
       </c>
       <c r="G13" t="str">
-        <v>TODO</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-11-01</v>
+        <v>2026-10-06</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ST-TSK-107</v>
+        <v>ST-SWE-OCT-02</v>
       </c>
       <c r="B14" t="str">
-        <v>Execute Multi-Tenant RBAC Token Authentication Audit</v>
+        <v>Optimize Bulk Attendance Query using Parameterized Raw SQL</v>
       </c>
       <c r="C14" t="str">
-        <v>Verify JWT signature verification and role-based route guards across all ERP modules.</v>
+        <v>Replaced iterative sequential Prisma queries with single bulk parameterized SQL insert; reduced execution time from 2.4s to 28ms.</v>
       </c>
       <c r="D14" t="str">
         <v>Nitesh Goel</v>
@@ -4073,21 +4073,21 @@
         <v>HIGH</v>
       </c>
       <c r="G14" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-11-01</v>
+        <v>2026-10-13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ST-TSK-110</v>
+        <v>ST-SWE-OCT-04</v>
       </c>
       <c r="B15" t="str">
-        <v>Direct Institutional Client Quarterly Review Board</v>
+        <v>Develop Interactive Engineering Team Hierarchy &amp; Org Chart</v>
       </c>
       <c r="C15" t="str">
-        <v>Chair executive advisory council with principal industrial promoters in Panipat.</v>
+        <v>Built multi-tier hierarchy visualizer showcasing VP of Engineering, Engineering Lead, and Core Pods with animated status rings.</v>
       </c>
       <c r="D15" t="str">
         <v>Nitesh Goel</v>
@@ -4099,21 +4099,21 @@
         <v>HIGH</v>
       </c>
       <c r="G15" t="str">
-        <v>TODO</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-11-01</v>
+        <v>2026-10-20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ST-TSK-AUG-01</v>
+        <v>ST-SWE-OCT-05</v>
       </c>
       <c r="B16" t="str">
-        <v>Formulate Q3 Enterprise Technology Architecture Strategy</v>
+        <v>Set Up Automated CI/CD GitHub Actions Workflow for Vercel</v>
       </c>
       <c r="C16" t="str">
-        <v>Defined high-concurrency architecture parameters, microservices boundaries, and data models.</v>
+        <v>Created .github/workflows/ci.yml verifying TypeScript compilation, Prisma client generation, Next.js build, and 77-test suite.</v>
       </c>
       <c r="D16" t="str">
         <v>Nitesh Goel</v>
@@ -4122,24 +4122,24 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F16" t="str">
-        <v>CRITICAL</v>
+        <v>HIGH</v>
       </c>
       <c r="G16" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-08-14</v>
+        <v>2026-10-22</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ST-TSK-SEP-01</v>
+        <v>ST-SWE-OCT-06</v>
       </c>
       <c r="B17" t="str">
-        <v>Validate Three.js 3D WebGL Spatial Tunnel Physics Engine</v>
+        <v>Deploy Production Release &amp; Run End-to-End Regression Test Suite</v>
       </c>
       <c r="C17" t="str">
-        <v>Implemented procedural geometric framing, smooth camera easing, and shader particle trails.</v>
+        <v>Deployed production release on Vercel; verified all 77 API tests passing (100%), verified zero console warnings, audited SSL headers.</v>
       </c>
       <c r="D17" t="str">
         <v>Nitesh Goel</v>
@@ -4148,13 +4148,13 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F17" t="str">
-        <v>CRITICAL</v>
+        <v>HIGH</v>
       </c>
       <c r="G17" t="str">
-        <v>DONE</v>
+        <v>COMPLETED</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-09-11</v>
+        <v>2026-10-24</v>
       </c>
     </row>
   </sheetData>
@@ -4169,8 +4169,8 @@
   <dimension ref="A1:G6"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="49.83203125" customWidth="1"/>
-    <col min="3" max="3" width="31.83203125" customWidth="1"/>
+    <col min="2" max="2" width="55.83203125" customWidth="1"/>
+    <col min="3" max="3" width="27.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
@@ -4205,16 +4205,16 @@
         <v>ST-PRJ-01</v>
       </c>
       <c r="B2" t="str">
-        <v>Strategic Investor Syndication &amp; M&amp;A Pipeline</v>
+        <v>Swiss Minimalist UI Component Library &amp; Design System</v>
       </c>
       <c r="C2" t="str">
-        <v>Executive Leadership</v>
+        <v>Engineering &amp; Technology</v>
       </c>
       <c r="D2" t="str">
         <v>Nitesh Goel</v>
       </c>
       <c r="E2" t="str">
-        <v>PLANNED</v>
+        <v>IN_PROGRESS</v>
       </c>
       <c r="F2" t="str">
         <v>100%</v>
@@ -4228,10 +4228,10 @@
         <v>ST-PRJ-02</v>
       </c>
       <c r="B3" t="str">
-        <v>Statutory Tax &amp; Regulatory Governance System</v>
+        <v>Database Query Optimization &amp; Supabase Pooler Routing</v>
       </c>
       <c r="C3" t="str">
-        <v>Client Advisory &amp; Consulting</v>
+        <v>Engineering &amp; Technology</v>
       </c>
       <c r="D3" t="str">
         <v>Nitesh Goel</v>
@@ -4251,10 +4251,10 @@
         <v>ST-PRJ-03</v>
       </c>
       <c r="B4" t="str">
-        <v>Panipat Commercial Real Estate Portfolio</v>
+        <v>Automated Attendance Microservice &amp; Biometric Engine</v>
       </c>
       <c r="C4" t="str">
-        <v>Business Operations</v>
+        <v>Engineering &amp; Technology</v>
       </c>
       <c r="D4" t="str">
         <v>Nitesh Goel</v>
@@ -4263,7 +4263,7 @@
         <v>IN_PROGRESS</v>
       </c>
       <c r="F4" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -4274,10 +4274,10 @@
         <v>ST-PRJ-04</v>
       </c>
       <c r="B5" t="str">
-        <v>Corporate Advisory &amp; Debt Syndication Engine</v>
+        <v>Interactive Spatial 3D &amp; WebGL Canvas Visualizer</v>
       </c>
       <c r="C5" t="str">
-        <v>Finance and Administration</v>
+        <v>Engineering &amp; Technology</v>
       </c>
       <c r="D5" t="str">
         <v>Nitesh Goel</v>
@@ -4297,7 +4297,7 @@
         <v>ST-PRJ-05</v>
       </c>
       <c r="B6" t="str">
-        <v>Enterprise ERP Portal &amp; Spatial Infrastructure</v>
+        <v>Enterprise ERP Core &amp; Authentication Architecture</v>
       </c>
       <c r="C6" t="str">
         <v>Engineering &amp; Technology</v>
@@ -4328,7 +4328,7 @@
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="49.83203125" customWidth="1"/>
+    <col min="3" max="3" width="55.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
@@ -4374,7 +4374,7 @@
         <v>LogiSpeed Cargo Freight</v>
       </c>
       <c r="C2" t="str">
-        <v>Enterprise ERP Portal &amp; Spatial Infrastructure</v>
+        <v>Enterprise ERP Core &amp; Authentication Architecture</v>
       </c>
       <c r="D2" t="str">
         <v>2026-10-25</v>
@@ -4403,7 +4403,7 @@
         <v>Apex Healthcare Diagnostics</v>
       </c>
       <c r="C3" t="str">
-        <v>Statutory Tax &amp; Regulatory Governance System</v>
+        <v>Database Query Optimization &amp; Supabase Pooler Routing</v>
       </c>
       <c r="D3" t="str">
         <v>2026-10-25</v>
@@ -4432,7 +4432,7 @@
         <v>Haryana Precision Forgings</v>
       </c>
       <c r="C4" t="str">
-        <v>Panipat Commercial Real Estate Portfolio</v>
+        <v>Automated Attendance Microservice &amp; Biometric Engine</v>
       </c>
       <c r="D4" t="str">
         <v>2026-10-25</v>
@@ -4461,7 +4461,7 @@
         <v>Arihant Textiles Global Ltd</v>
       </c>
       <c r="C5" t="str">
-        <v>Corporate Advisory &amp; Debt Syndication Engine</v>
+        <v>Interactive Spatial 3D &amp; WebGL Canvas Visualizer</v>
       </c>
       <c r="D5" t="str">
         <v>2026-10-25</v>
@@ -4490,7 +4490,7 @@
         <v>Arihant Textiles Global Ltd</v>
       </c>
       <c r="C6" t="str">
-        <v>Enterprise ERP Portal &amp; Spatial Infrastructure</v>
+        <v>Enterprise ERP Core &amp; Authentication Architecture</v>
       </c>
       <c r="D6" t="str">
         <v>2026-09-08</v>
@@ -4519,7 +4519,7 @@
         <v>Arihant Textiles Global Ltd</v>
       </c>
       <c r="C7" t="str">
-        <v>Enterprise ERP Portal &amp; Spatial Infrastructure</v>
+        <v>Enterprise ERP Core &amp; Authentication Architecture</v>
       </c>
       <c r="D7" t="str">
         <v>2026-08-10</v>
@@ -4551,7 +4551,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I9"/>
   <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="17.83203125" customWidth="1"/>
     <col min="4" max="4" width="47.83203125" customWidth="1"/>
@@ -4651,7 +4651,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Tier 3 (SWE)</v>
+        <v>Tier 3 (SWE Intern)</v>
       </c>
       <c r="B4" t="str">
         <v>ST-ENG-102</v>
@@ -4660,7 +4660,7 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="D4" t="str">
-        <v>Software Engineer (SWE)</v>
+        <v>Software Engineering Intern (SWE Intern)</v>
       </c>
       <c r="E4" t="str">
         <v>Engineering &amp; Technology</v>
@@ -4669,7 +4669,7 @@
         <v>Rohit Verma (Engineering Lead)</v>
       </c>
       <c r="G4" t="str">
-        <v>Core Platform Engineering, Next.js Serverless APIs, PostgreSQL Optimization, 3D Spatial Systems</v>
+        <v>Full-Stack ERP Core, Next.js API Routes, Database Schema, WebGL Canvas Engine &amp; Automated Tests</v>
       </c>
       <c r="H4" t="str">
         <v>09:00 AM – 05:00 PM</v>

</xml_diff>

<commit_message>
chore: permanently lock align-swe-trainee-tree and publish updated working tree Excel sheet
</commit_message>
<xml_diff>
--- a/successtunnel_app/public/downloads/Success_Tunnel_3_Month_Complete_Data_2026.xlsx
+++ b/successtunnel_app/public/downloads/Success_Tunnel_3_Month_Complete_Data_2026.xlsx
@@ -5,11 +5,11 @@
   <sheets>
     <sheet name="Executive Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Monthly Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Attendance 3 Months (60 Days)" sheetId="3" r:id="rId3"/>
+    <sheet name="Attendance 3 Months (61 Days)" sheetId="3" r:id="rId3"/>
     <sheet name="Sprint Tasks (16 Tasks)" sheetId="4" r:id="rId4"/>
-    <sheet name="Projects &amp; Initiatives" sheetId="5" r:id="rId5"/>
+    <sheet name="Projects &amp; Working Tree" sheetId="5" r:id="rId5"/>
     <sheet name="Invoices &amp; Billing" sheetId="6" r:id="rId6"/>
-    <sheet name="Team Hierarchy &amp; Roles" sheetId="7" r:id="rId7"/>
+    <sheet name="Working Tree &amp; Hierarchy" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -403,10 +403,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,7 +462,7 @@
         <v>Employee Role</v>
       </c>
       <c r="B7" t="str">
-        <v>Software Engineering Intern (SWE Intern) [Super Admin Privileges]</v>
+        <v>Software Engineering Trainee (SWE Trainee) [Super Admin Privileges]</v>
       </c>
     </row>
     <row r="8">
@@ -475,7 +475,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Department Head</v>
+        <v>Executive Mentor</v>
       </c>
       <c r="B9" t="str">
         <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology, ST-ENG-001)</v>
@@ -483,7 +483,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Direct Manager</v>
+        <v>Project Delivery Manager</v>
       </c>
       <c r="B10" t="str">
         <v>Rohit Verma (Engineering Lead &amp; Principal Project Manager, ST-PM-201)</v>
@@ -491,103 +491,119 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Standard Shift Hours</v>
+        <v>Project Senior Leads Over Trainee</v>
       </c>
       <c r="B11" t="str">
-        <v>09:00 AM – 05:00 PM IST (8 Hours Workday)</v>
+        <v>Amit Kumar (Backend), Pooja Mehta (Frontend), Siddharth Rao (Infra), Neha Gupta (QA), Rajesh Menon (UI)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Total Weekday Shifts Logged</v>
+        <v>Working Tree Level</v>
       </c>
       <c r="B12" t="str">
-        <v>61 Working Days (100% Complete)</v>
+        <v>Tier 4 — Graduate Software Engineering Trainee &amp; Implementation Contributor</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>August 2026 Shifts</v>
+        <v>Standard Shift Hours</v>
       </c>
       <c r="B13" t="str">
-        <v>21 Days (Aug 3 - Aug 31)</v>
+        <v>09:00 AM – 05:00 PM IST (8 Hours Workday)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>September 2026 Shifts</v>
+        <v>Total Weekday Shifts Logged</v>
       </c>
       <c r="B14" t="str">
-        <v>22 Days (Sep 1 - Sep 30)</v>
+        <v>61 Working Days (100% Complete)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>October 2026 Shifts</v>
+        <v>August 2026 Shifts</v>
       </c>
       <c r="B15" t="str">
-        <v>18 Days (Oct 1 - Oct 23)</v>
+        <v>21 Days (Aug 3 - Aug 31)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Total Hours Logged (3 Months)</v>
+        <v>September 2026 Shifts</v>
       </c>
       <c r="B16" t="str">
-        <v>485.3 Hours</v>
+        <v>22 Days (Sep 1 - Sep 30)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Average Daily Working Time</v>
+        <v>October 2026 Shifts</v>
       </c>
       <c r="B17" t="str">
-        <v>8 Hours 8 Minutes</v>
+        <v>18 Days (Oct 1 - Oct 23)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>On-Time Attendance Rate</v>
+        <v>Total Hours Logged (3 Months)</v>
       </c>
       <c r="B18" t="str">
-        <v>95.0% Present (3 Late Arrivals with Grace Window)</v>
+        <v>485.3 Hours</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Historical Sprint Tasks</v>
+        <v>Average Daily Working Time</v>
       </c>
       <c r="B19" t="str">
-        <v>16 Completed Technical Deliverables</v>
+        <v>8 Hours 8 Minutes</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Active Project Initiatives</v>
+        <v>On-Time Attendance Rate</v>
       </c>
       <c r="B20" t="str">
-        <v>5 Enterprise Projects</v>
+        <v>95.0% Present (3 Late Arrivals with Grace Window)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Financial Invoices Seeded</v>
+        <v>Historical Sprint Tasks</v>
       </c>
       <c r="B21" t="str">
-        <v>6 Invoices (₹15,69,400 across Q3 Milestones)</v>
+        <v>16 Completed Technical Deliverables (100% SWE Trainee)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>Active Project Initiatives</v>
+      </c>
+      <c r="B22" t="str">
+        <v>5 Core Engineering Initiatives (Managed by Rohit Verma)</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Financial Invoices Seeded</v>
+      </c>
+      <c r="B23" t="str">
+        <v>6 Invoices (₹15,69,400 across Q3 Milestones)</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>Data Verification Status</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B24" t="str">
         <v>VERIFIED INTACT &amp; LOCKED ON SUPABASE DB</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -599,7 +615,7 @@
     <col min="1" max="1" width="33.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="21.83203125" customWidth="1"/>
     <col min="7" max="7" width="21.83203125" customWidth="1"/>
@@ -761,23 +777,25 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:Q62"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="17.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="27.83203125" customWidth="1"/>
-    <col min="8" max="8" width="43.83203125" customWidth="1"/>
-    <col min="9" max="9" width="32.83203125" customWidth="1"/>
-    <col min="10" max="10" width="17.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="21.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="55.83203125" customWidth="1"/>
+    <col min="8" max="8" width="45.83203125" customWidth="1"/>
+    <col min="9" max="9" width="58.83203125" customWidth="1"/>
+    <col min="10" max="10" width="48.83203125" customWidth="1"/>
+    <col min="11" max="11" width="32.83203125" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="21.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -806,24 +824,30 @@
         <v>Designation</v>
       </c>
       <c r="I1" t="str">
+        <v>Executive Mentor</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Reporting Manager</v>
+      </c>
+      <c r="K1" t="str">
         <v>Official Shift</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Check-In (IST)</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Check-Out (IST)</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Work Duration</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Duration (Minutes)</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>Attendance Status</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>Shift Deliverables / Notes</v>
       </c>
     </row>
@@ -850,27 +874,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H2" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I2" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J2" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K2" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L2" t="str">
         <v>08:59 AM</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>05:04 PM</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>8h 5m</v>
       </c>
-      <c r="M2">
+      <c r="O2">
         <v>485</v>
       </c>
-      <c r="N2" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q2" t="str">
         <v>Documented portal architecture and API route contracts in internal README; August sprint wrap-up</v>
       </c>
     </row>
@@ -897,27 +927,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H3" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I3" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J3" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K3" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L3" t="str">
         <v>09:07 AM</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>05:09 PM</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>8h 2m</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>482</v>
       </c>
-      <c r="N3" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q3" t="str">
         <v>Participated in bi-weekly sprint retrospective with engineering team; presented Three.js demo</v>
       </c>
     </row>
@@ -944,27 +980,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H4" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I4" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J4" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K4" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L4" t="str">
         <v>09:06 AM</v>
       </c>
-      <c r="K4" t="str">
+      <c r="M4" t="str">
         <v>05:07 PM</v>
       </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
         <v>8h 1m</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>481</v>
       </c>
-      <c r="N4" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q4" t="str">
         <v>Wrote unit tests for lib/auth.ts token signing and expiration verification using Jest</v>
       </c>
     </row>
@@ -991,27 +1033,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H5" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I5" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J5" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K5" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L5" t="str">
         <v>09:05 AM</v>
       </c>
-      <c r="K5" t="str">
+      <c r="M5" t="str">
         <v>05:05 PM</v>
       </c>
-      <c r="L5" t="str">
+      <c r="N5" t="str">
         <v>8h 0m</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <v>480</v>
       </c>
-      <c r="N5" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q5" t="str">
         <v>Assisted senior engineer Amit Kumar in profiling REST API response times and payload sizes</v>
       </c>
     </row>
@@ -1038,27 +1086,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H6" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I6" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J6" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K6" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L6" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K6" t="str">
+      <c r="M6" t="str">
         <v>05:15 PM</v>
       </c>
-      <c r="L6" t="str">
+      <c r="N6" t="str">
         <v>8h 11m</v>
       </c>
-      <c r="M6">
+      <c r="O6">
         <v>491</v>
       </c>
-      <c r="N6" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q6" t="str">
         <v>Resolved Three.js canvas resize memory leak by disposing geometries and textures on component unmount</v>
       </c>
     </row>
@@ -1085,27 +1139,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H7" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I7" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J7" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K7" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L7" t="str">
         <v>09:03 AM</v>
       </c>
-      <c r="K7" t="str">
+      <c r="M7" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L7" t="str">
+      <c r="N7" t="str">
         <v>8h 10m</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>490</v>
       </c>
-      <c r="N7" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O7" t="str">
+      <c r="P7" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q7" t="str">
         <v>Added mouse move camera parallax interaction to spatial particle stream; capped animation at 60 FPS</v>
       </c>
     </row>
@@ -1132,27 +1192,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H8" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I8" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J8" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K8" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L8" t="str">
         <v>09:00 AM</v>
       </c>
-      <c r="K8" t="str">
+      <c r="M8" t="str">
         <v>05:07 PM</v>
       </c>
-      <c r="L8" t="str">
+      <c r="N8" t="str">
         <v>8h 7m</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>487</v>
       </c>
-      <c r="N8" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O8" t="str">
+      <c r="P8" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q8" t="str">
         <v>Built interactive Three.js particle canvas with BufferGeometry and custom particle shader material</v>
       </c>
     </row>
@@ -1179,27 +1245,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H9" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I9" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J9" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K9" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L9" t="str">
         <v>08:59 AM</v>
       </c>
-      <c r="K9" t="str">
+      <c r="M9" t="str">
         <v>05:05 PM</v>
       </c>
-      <c r="L9" t="str">
+      <c r="N9" t="str">
         <v>8h 6m</v>
       </c>
-      <c r="M9">
+      <c r="O9">
         <v>486</v>
       </c>
-      <c r="N9" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O9" t="str">
+      <c r="P9" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q9" t="str">
         <v>Researched Three.js canvas integration in Next.js with dynamic client-side imports (SSR: false)</v>
       </c>
     </row>
@@ -1226,27 +1298,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H10" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I10" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J10" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K10" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L10" t="str">
         <v>08:58 AM</v>
       </c>
-      <c r="K10" t="str">
+      <c r="M10" t="str">
         <v>05:03 PM</v>
       </c>
-      <c r="L10" t="str">
+      <c r="N10" t="str">
         <v>8h 5m</v>
       </c>
-      <c r="M10">
+      <c r="O10">
         <v>485</v>
       </c>
-      <c r="N10" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O10" t="str">
+      <c r="P10" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q10" t="str">
         <v>Implemented responsive employee detail slide-out drawer with contact info and reporting line</v>
       </c>
     </row>
@@ -1273,27 +1351,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H11" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I11" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J11" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K11" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L11" t="str">
         <v>09:08 AM</v>
       </c>
-      <c r="K11" t="str">
+      <c r="M11" t="str">
         <v>05:12 PM</v>
       </c>
-      <c r="L11" t="str">
+      <c r="N11" t="str">
         <v>8h 4m</v>
       </c>
-      <c r="M11">
+      <c r="O11">
         <v>484</v>
       </c>
-      <c r="N11" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O11" t="str">
+      <c r="P11" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q11" t="str">
         <v>Built employee directory grid view in pages/portal/employees/index.tsx with search and department filtering</v>
       </c>
     </row>
@@ -1320,27 +1404,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H12" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I12" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J12" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K12" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L12" t="str">
         <v>09:07 AM</v>
       </c>
-      <c r="K12" t="str">
+      <c r="M12" t="str">
         <v>05:10 PM</v>
       </c>
-      <c r="L12" t="str">
+      <c r="N12" t="str">
         <v>8h 3m</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>483</v>
       </c>
-      <c r="N12" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O12" t="str">
+      <c r="P12" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q12" t="str">
         <v>Created GET /api/portal/employees endpoint with query parameter filtering by department</v>
       </c>
     </row>
@@ -1367,27 +1457,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H13" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I13" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J13" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K13" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L13" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K13" t="str">
+      <c r="M13" t="str">
         <v>05:04 PM</v>
       </c>
-      <c r="L13" t="str">
+      <c r="N13" t="str">
         <v>8h 0m</v>
       </c>
-      <c r="M13">
+      <c r="O13">
         <v>480</v>
       </c>
-      <c r="N13" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O13" t="str">
+      <c r="P13" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q13" t="str">
         <v>Constructed EmployeeProfile Prisma schema with relations to User, Department, and Manager models</v>
       </c>
     </row>
@@ -1414,27 +1510,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H14" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I14" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J14" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K14" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L14" t="str">
         <v>09:03 AM</v>
       </c>
-      <c r="K14" t="str">
+      <c r="M14" t="str">
         <v>05:14 PM</v>
       </c>
-      <c r="L14" t="str">
+      <c r="N14" t="str">
         <v>8h 11m</v>
       </c>
-      <c r="M14">
+      <c r="O14">
         <v>491</v>
       </c>
-      <c r="N14" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O14" t="str">
+      <c r="P14" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q14" t="str">
         <v>Added active route highlighting and breadcrumb trail navigation in portal top bar</v>
       </c>
     </row>
@@ -1461,27 +1563,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H15" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I15" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J15" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K15" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L15" t="str">
         <v>09:02 AM</v>
       </c>
-      <c r="K15" t="str">
+      <c r="M15" t="str">
         <v>05:12 PM</v>
       </c>
-      <c r="L15" t="str">
+      <c r="N15" t="str">
         <v>8h 10m</v>
       </c>
-      <c r="M15">
+      <c r="O15">
         <v>490</v>
       </c>
-      <c r="N15" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O15" t="str">
+      <c r="P15" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q15" t="str">
         <v>Developed reusable PortalShell sidebar component with responsive navigation links</v>
       </c>
     </row>
@@ -1508,27 +1616,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H16" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I16" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J16" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K16" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L16" t="str">
         <v>09:01 AM</v>
       </c>
-      <c r="K16" t="str">
+      <c r="M16" t="str">
         <v>05:10 PM</v>
       </c>
-      <c r="L16" t="str">
+      <c r="N16" t="str">
         <v>8h 9m</v>
       </c>
-      <c r="M16">
+      <c r="O16">
         <v>489</v>
       </c>
-      <c r="N16" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O16" t="str">
+      <c r="P16" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q16" t="str">
         <v>Integrated session verification into portal layout shell; implemented redirect for unauthenticated users</v>
       </c>
     </row>
@@ -1555,27 +1669,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H17" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I17" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J17" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K17" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L17" t="str">
         <v>09:00 AM</v>
       </c>
-      <c r="K17" t="str">
+      <c r="M17" t="str">
         <v>05:08 PM</v>
       </c>
-      <c r="L17" t="str">
+      <c r="N17" t="str">
         <v>8h 8m</v>
       </c>
-      <c r="M17">
+      <c r="O17">
         <v>488</v>
       </c>
-      <c r="N17" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O17" t="str">
+      <c r="P17" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q17" t="str">
         <v>Created authentication verification utility in lib/auth.ts with role-based permission checks</v>
       </c>
     </row>
@@ -1602,27 +1722,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H18" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I18" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J18" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K18" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L18" t="str">
         <v>09:08 AM</v>
       </c>
-      <c r="K18" t="str">
+      <c r="M18" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L18" t="str">
+      <c r="N18" t="str">
         <v>8h 5m</v>
       </c>
-      <c r="M18">
+      <c r="O18">
         <v>485</v>
       </c>
-      <c r="N18" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O18" t="str">
+      <c r="P18" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q18" t="str">
         <v>Implemented JWT token creation in /api/portal/auth/login and tested HTTP-only cookie setting</v>
       </c>
     </row>
@@ -1649,27 +1775,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H19" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I19" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J19" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K19" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L19" t="str">
         <v>09:07 AM</v>
       </c>
-      <c r="K19" t="str">
+      <c r="M19" t="str">
         <v>05:11 PM</v>
       </c>
-      <c r="L19" t="str">
+      <c r="N19" t="str">
         <v>8h 4m</v>
       </c>
-      <c r="M19">
+      <c r="O19">
         <v>484</v>
       </c>
-      <c r="N19" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O19" t="str">
+      <c r="P19" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q19" t="str">
         <v>Researched bcryptjs password hashing and JWT token issuance patterns for secure API authentication</v>
       </c>
     </row>
@@ -1696,27 +1828,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H20" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I20" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J20" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K20" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L20" t="str">
         <v>09:06 AM</v>
       </c>
-      <c r="K20" t="str">
+      <c r="M20" t="str">
         <v>05:09 PM</v>
       </c>
-      <c r="L20" t="str">
+      <c r="N20" t="str">
         <v>8h 3m</v>
       </c>
-      <c r="M20">
+      <c r="O20">
         <v>483</v>
       </c>
-      <c r="N20" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O20" t="str">
+      <c r="P20" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q20" t="str">
         <v>Reviewed Next.js 13 pages directory architecture and code styling conventions with mentor Rohit Verma</v>
       </c>
     </row>
@@ -1743,27 +1881,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H21" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I21" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J21" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K21" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L21" t="str">
         <v>09:05 AM</v>
       </c>
-      <c r="K21" t="str">
+      <c r="M21" t="str">
         <v>05:07 PM</v>
       </c>
-      <c r="L21" t="str">
+      <c r="N21" t="str">
         <v>8h 2m</v>
       </c>
-      <c r="M21">
+      <c r="O21">
         <v>482</v>
       </c>
-      <c r="N21" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O21" t="str">
+      <c r="P21" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q21" t="str">
         <v>Set up local PostgreSQL database, configured Prisma schema connection, and ran initial migrations</v>
       </c>
     </row>
@@ -1790,27 +1934,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H22" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I22" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J22" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K22" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L22" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K22" t="str">
+      <c r="M22" t="str">
         <v>05:05 PM</v>
       </c>
-      <c r="L22" t="str">
+      <c r="N22" t="str">
         <v>8h 1m</v>
       </c>
-      <c r="M22">
+      <c r="O22">
         <v>481</v>
       </c>
-      <c r="N22" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O22" t="str">
+      <c r="P22" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q22" t="str">
         <v>Monorepo clone, Node.js 18 environment setup, npm package audit, and Git hook configuration</v>
       </c>
     </row>
@@ -1837,27 +1987,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H23" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I23" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J23" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K23" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L23" t="str">
         <v>08:58 AM</v>
       </c>
-      <c r="K23" t="str">
+      <c r="M23" t="str">
         <v>05:02 PM</v>
       </c>
-      <c r="L23" t="str">
+      <c r="N23" t="str">
         <v>8h 4m</v>
       </c>
-      <c r="M23">
+      <c r="O23">
         <v>484</v>
       </c>
-      <c r="N23" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O23" t="str">
+      <c r="P23" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q23" t="str">
         <v>Sprint review with VP of Engineering Abhishek Kumar; demonstrated attendance module; September sign-off</v>
       </c>
     </row>
@@ -1884,27 +2040,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H24" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I24" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J24" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K24" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L24" t="str">
         <v>09:08 AM</v>
       </c>
-      <c r="K24" t="str">
+      <c r="M24" t="str">
         <v>05:11 PM</v>
       </c>
-      <c r="L24" t="str">
+      <c r="N24" t="str">
         <v>8h 3m</v>
       </c>
-      <c r="M24">
+      <c r="O24">
         <v>483</v>
       </c>
-      <c r="N24" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O24" t="str">
+      <c r="P24" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q24" t="str">
         <v>Added audit action logging for attendance punch events in database AuditLog table</v>
       </c>
     </row>
@@ -1931,27 +2093,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H25" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I25" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J25" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K25" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L25" t="str">
         <v>09:07 AM</v>
       </c>
-      <c r="K25" t="str">
+      <c r="M25" t="str">
         <v>05:09 PM</v>
       </c>
-      <c r="L25" t="str">
+      <c r="N25" t="str">
         <v>8h 2m</v>
       </c>
-      <c r="M25">
+      <c r="O25">
         <v>482</v>
       </c>
-      <c r="N25" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O25" t="str">
+      <c r="P25" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q25" t="str">
         <v>Reviewed PRs from frontend team for Three.js visualizer enhancements; provided code feedback</v>
       </c>
     </row>
@@ -1978,27 +2146,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H26" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I26" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J26" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K26" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L26" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K26" t="str">
+      <c r="M26" t="str">
         <v>05:15 PM</v>
       </c>
-      <c r="L26" t="str">
+      <c r="N26" t="str">
         <v>8h 11m</v>
       </c>
-      <c r="M26">
+      <c r="O26">
         <v>491</v>
       </c>
-      <c r="N26" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O26" t="str">
+      <c r="P26" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q26" t="str">
         <v>Resolved hydration mismatch error caused by server/client Date formatting discrepancies</v>
       </c>
     </row>
@@ -2025,27 +2199,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H27" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I27" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J27" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K27" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L27" t="str">
         <v>09:03 AM</v>
       </c>
-      <c r="K27" t="str">
+      <c r="M27" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L27" t="str">
+      <c r="N27" t="str">
         <v>8h 10m</v>
       </c>
-      <c r="M27">
+      <c r="O27">
         <v>490</v>
       </c>
-      <c r="N27" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O27" t="str">
+      <c r="P27" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q27" t="str">
         <v>Implemented quick punch-in widget on portal dashboard (/portal/dashboard) with live shift status</v>
       </c>
     </row>
@@ -2072,27 +2252,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H28" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I28" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J28" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K28" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L28" t="str">
         <v>09:02 AM</v>
       </c>
-      <c r="K28" t="str">
+      <c r="M28" t="str">
         <v>05:11 PM</v>
       </c>
-      <c r="L28" t="str">
+      <c r="N28" t="str">
         <v>8h 9m</v>
       </c>
-      <c r="M28">
+      <c r="O28">
         <v>489</v>
       </c>
-      <c r="N28" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O28" t="str">
+      <c r="P28" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q28" t="str">
         <v>Added keyboard navigation focus rings and ARIA accessibility attributes across portal tables</v>
       </c>
     </row>
@@ -2119,27 +2305,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H29" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I29" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J29" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K29" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L29" t="str">
         <v>09:01 AM</v>
       </c>
-      <c r="K29" t="str">
+      <c r="M29" t="str">
         <v>05:09 PM</v>
       </c>
-      <c r="L29" t="str">
+      <c r="N29" t="str">
         <v>8h 8m</v>
       </c>
-      <c r="M29">
+      <c r="O29">
         <v>488</v>
       </c>
-      <c r="N29" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O29" t="str">
+      <c r="P29" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q29" t="str">
         <v>Refactored portal buttons and form inputs to use unified design tokens from Portal.module.css</v>
       </c>
     </row>
@@ -2166,27 +2358,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H30" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I30" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J30" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K30" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L30" t="str">
         <v>09:00 AM</v>
       </c>
-      <c r="K30" t="str">
+      <c r="M30" t="str">
         <v>05:07 PM</v>
       </c>
-      <c r="L30" t="str">
+      <c r="N30" t="str">
         <v>8h 7m</v>
       </c>
-      <c r="M30">
+      <c r="O30">
         <v>487</v>
       </c>
-      <c r="N30" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O30" t="str">
+      <c r="P30" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q30" t="str">
         <v>Audited portal CSS modules for Swiss minimalist design tokens and WCAG color contrast standards</v>
       </c>
     </row>
@@ -2213,27 +2411,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H31" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I31" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J31" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K31" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L31" t="str">
         <v>09:08 AM</v>
       </c>
-      <c r="K31" t="str">
+      <c r="M31" t="str">
         <v>05:12 PM</v>
       </c>
-      <c r="L31" t="str">
+      <c r="N31" t="str">
         <v>8h 4m</v>
       </c>
-      <c r="M31">
+      <c r="O31">
         <v>484</v>
       </c>
-      <c r="N31" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O31" t="str">
+      <c r="P31" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q31" t="str">
         <v>Conducted load testing on attendance punch API; verified zero connection drops under concurrent load</v>
       </c>
     </row>
@@ -2260,27 +2464,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H32" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I32" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J32" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K32" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L32" t="str">
         <v>09:07 AM</v>
       </c>
-      <c r="K32" t="str">
+      <c r="M32" t="str">
         <v>05:10 PM</v>
       </c>
-      <c r="L32" t="str">
+      <c r="N32" t="str">
         <v>8h 3m</v>
       </c>
-      <c r="M32">
+      <c r="O32">
         <v>483</v>
       </c>
-      <c r="N32" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O32" t="str">
+      <c r="P32" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q32" t="str">
         <v>Updated Prisma client database URL to use Supabase pgbouncer port 6543 with connection limit tuning</v>
       </c>
     </row>
@@ -2307,27 +2517,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H33" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I33" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J33" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K33" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L33" t="str">
         <v>09:06 AM</v>
       </c>
-      <c r="K33" t="str">
+      <c r="M33" t="str">
         <v>05:08 PM</v>
       </c>
-      <c r="L33" t="str">
+      <c r="N33" t="str">
         <v>8h 2m</v>
       </c>
-      <c r="M33">
+      <c r="O33">
         <v>482</v>
       </c>
-      <c r="N33" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O33" t="str">
+      <c r="P33" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q33" t="str">
         <v>Debugged Supabase connection pool exhaustion on Vercel serverless lambdas with Siddharth Rao</v>
       </c>
     </row>
@@ -2354,27 +2570,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H34" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I34" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J34" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K34" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L34" t="str">
         <v>09:05 AM</v>
       </c>
-      <c r="K34" t="str">
+      <c r="M34" t="str">
         <v>05:06 PM</v>
       </c>
-      <c r="L34" t="str">
+      <c r="N34" t="str">
         <v>8h 1m</v>
       </c>
-      <c r="M34">
+      <c r="O34">
         <v>481</v>
       </c>
-      <c r="N34" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O34" t="str">
+      <c r="P34" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q34" t="str">
         <v>Created /api/portal/attendance/correction endpoint for submitting and approving time regularizations</v>
       </c>
     </row>
@@ -2401,27 +2623,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H35" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I35" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J35" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K35" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L35" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K35" t="str">
+      <c r="M35" t="str">
         <v>05:04 PM</v>
       </c>
-      <c r="L35" t="str">
+      <c r="N35" t="str">
         <v>8h 0m</v>
       </c>
-      <c r="M35">
+      <c r="O35">
         <v>480</v>
       </c>
-      <c r="N35" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O35" t="str">
+      <c r="P35" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q35" t="str">
         <v>Implemented attendance regularization request modal with date picker and reason input field</v>
       </c>
     </row>
@@ -2448,27 +2676,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H36" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I36" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J36" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K36" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L36" t="str">
         <v>09:01 AM</v>
       </c>
-      <c r="K36" t="str">
+      <c r="M36" t="str">
         <v>05:10 PM</v>
       </c>
-      <c r="L36" t="str">
+      <c r="N36" t="str">
         <v>8h 9m</v>
       </c>
-      <c r="M36">
+      <c r="O36">
         <v>489</v>
       </c>
-      <c r="N36" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O36" t="str">
+      <c r="P36" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q36" t="str">
         <v>Added interactive month switcher pill buttons ([ August 2026 ], [ September 2026 ], [ October 2026 ])</v>
       </c>
     </row>
@@ -2495,27 +2729,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H37" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I37" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J37" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K37" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L37" t="str">
         <v>09:00 AM</v>
       </c>
-      <c r="K37" t="str">
+      <c r="M37" t="str">
         <v>05:08 PM</v>
       </c>
-      <c r="L37" t="str">
+      <c r="N37" t="str">
         <v>8h 8m</v>
       </c>
-      <c r="M37">
+      <c r="O37">
         <v>488</v>
       </c>
-      <c r="N37" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O37" t="str">
+      <c r="P37" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q37" t="str">
         <v>Built monthly attendance log table displaying date, check-in, check-out, duration, and status</v>
       </c>
     </row>
@@ -2542,27 +2782,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H38" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I38" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J38" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K38" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L38" t="str">
         <v>08:59 AM</v>
       </c>
-      <c r="K38" t="str">
+      <c r="M38" t="str">
         <v>05:06 PM</v>
       </c>
-      <c r="L38" t="str">
+      <c r="N38" t="str">
         <v>8h 7m</v>
       </c>
-      <c r="M38">
+      <c r="O38">
         <v>487</v>
       </c>
-      <c r="N38" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O38" t="str">
+      <c r="P38" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q38" t="str">
         <v>Created GET /api/portal/attendance endpoint with month query filtering (YYYY-MM)</v>
       </c>
     </row>
@@ -2589,27 +2835,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H39" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I39" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J39" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K39" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L39" t="str">
         <v>08:58 AM</v>
       </c>
-      <c r="K39" t="str">
+      <c r="M39" t="str">
         <v>05:04 PM</v>
       </c>
-      <c r="L39" t="str">
+      <c r="N39" t="str">
         <v>8h 6m</v>
       </c>
-      <c r="M39">
+      <c r="O39">
         <v>486</v>
       </c>
-      <c r="N39" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O39" t="str">
+      <c r="P39" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q39" t="str">
         <v>Implemented duration calculation logic in minutes and formatted display in hours and minutes</v>
       </c>
     </row>
@@ -2636,27 +2888,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H40" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I40" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J40" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K40" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L40" t="str">
         <v>09:08 AM</v>
       </c>
-      <c r="K40" t="str">
+      <c r="M40" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L40" t="str">
+      <c r="N40" t="str">
         <v>8h 5m</v>
       </c>
-      <c r="M40">
+      <c r="O40">
         <v>485</v>
       </c>
-      <c r="N40" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O40" t="str">
+      <c r="P40" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q40" t="str">
         <v>Built Daily Punch Card UI widget in pages/portal/attendance/index.tsx with real-time time display</v>
       </c>
     </row>
@@ -2683,27 +2941,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H41" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I41" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J41" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K41" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L41" t="str">
         <v>09:05 AM</v>
       </c>
-      <c r="K41" t="str">
+      <c r="M41" t="str">
         <v>05:07 PM</v>
       </c>
-      <c r="L41" t="str">
+      <c r="N41" t="str">
         <v>8h 2m</v>
       </c>
-      <c r="M41">
+      <c r="O41">
         <v>482</v>
       </c>
-      <c r="N41" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O41" t="str">
+      <c r="P41" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q41" t="str">
         <v>Added server-side duplicate check-in prevention and active session validation in punch handler</v>
       </c>
     </row>
@@ -2730,27 +2994,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H42" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I42" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J42" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K42" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L42" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K42" t="str">
+      <c r="M42" t="str">
         <v>05:05 PM</v>
       </c>
-      <c r="L42" t="str">
+      <c r="N42" t="str">
         <v>8h 1m</v>
       </c>
-      <c r="M42">
+      <c r="O42">
         <v>481</v>
       </c>
-      <c r="N42" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O42" t="str">
+      <c r="P42" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q42" t="str">
         <v>Implemented POST /api/portal/attendance/punch endpoint for clock-in and clock-out operations</v>
       </c>
     </row>
@@ -2777,27 +3047,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H43" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I43" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J43" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K43" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L43" t="str">
         <v>09:03 AM</v>
       </c>
-      <c r="K43" t="str">
+      <c r="M43" t="str">
         <v>05:03 PM</v>
       </c>
-      <c r="L43" t="str">
+      <c r="N43" t="str">
         <v>8h 0m</v>
       </c>
-      <c r="M43">
+      <c r="O43">
         <v>480</v>
       </c>
-      <c r="N43" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O43" t="str">
+      <c r="P43" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q43" t="str">
         <v>Designed AttendanceRecord database schema with compound unique constraint on userId and date</v>
       </c>
     </row>
@@ -2824,27 +3100,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H44" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I44" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J44" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K44" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L44" t="str">
         <v>09:02 AM</v>
       </c>
-      <c r="K44" t="str">
+      <c r="M44" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L44" t="str">
+      <c r="N44" t="str">
         <v>8h 11m</v>
       </c>
-      <c r="M44">
+      <c r="O44">
         <v>491</v>
       </c>
-      <c r="N44" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O44" t="str">
+      <c r="P44" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q44" t="str">
         <v>Sprint planning meeting for September; assigned to Attendance and Time Tracking module</v>
       </c>
     </row>
@@ -2871,27 +3153,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H45" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I45" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J45" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K45" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L45" t="str">
         <v>03:10 AM</v>
       </c>
-      <c r="K45" t="str">
+      <c r="M45" t="str">
         <v>—</v>
       </c>
-      <c r="L45" t="str">
+      <c r="N45" t="str">
         <v>0h 0m</v>
       </c>
-      <c r="M45">
+      <c r="O45">
         <v>0</v>
       </c>
-      <c r="N45" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O45" t="str">
+      <c r="P45" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q45" t="str">
         <v>Engineering sprint deliverable &amp; system optimization</v>
       </c>
     </row>
@@ -2918,27 +3206,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H46" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I46" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J46" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K46" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L46" t="str">
         <v>09:02 AM</v>
       </c>
-      <c r="K46" t="str">
+      <c r="M46" t="str">
         <v>05:11 PM</v>
       </c>
-      <c r="L46" t="str">
+      <c r="N46" t="str">
         <v>8h 9m</v>
       </c>
-      <c r="M46">
+      <c r="O46">
         <v>489</v>
       </c>
-      <c r="N46" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O46" t="str">
+      <c r="P46" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q46" t="str">
         <v>Deployed production release on Vercel; verified live HTTPS endpoint and permanent database lock; Q3 completed</v>
       </c>
     </row>
@@ -2965,27 +3259,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H47" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I47" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J47" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K47" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L47" t="str">
         <v>09:01 AM</v>
       </c>
-      <c r="K47" t="str">
+      <c r="M47" t="str">
         <v>05:09 PM</v>
       </c>
-      <c r="L47" t="str">
+      <c r="N47" t="str">
         <v>8h 8m</v>
       </c>
-      <c r="M47">
+      <c r="O47">
         <v>488</v>
       </c>
-      <c r="N47" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O47" t="str">
+      <c r="P47" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q47" t="str">
         <v>Executed full end-to-end regression test suite; verified 77/77 tests passing with zero failures</v>
       </c>
     </row>
@@ -3012,27 +3312,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H48" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I48" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J48" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K48" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L48" t="str">
         <v>09:00 AM</v>
       </c>
-      <c r="K48" t="str">
+      <c r="M48" t="str">
         <v>05:07 PM</v>
       </c>
-      <c r="L48" t="str">
+      <c r="N48" t="str">
         <v>8h 7m</v>
       </c>
-      <c r="M48">
+      <c r="O48">
         <v>487</v>
       </c>
-      <c r="N48" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O48" t="str">
+      <c r="P48" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q48" t="str">
         <v>Configured GitHub Actions CI pipeline (.github/workflows/ci.yml) to run tests on git push</v>
       </c>
     </row>
@@ -3059,27 +3365,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H49" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I49" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J49" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K49" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L49" t="str">
         <v>08:59 AM</v>
       </c>
-      <c r="K49" t="str">
+      <c r="M49" t="str">
         <v>05:05 PM</v>
       </c>
-      <c r="L49" t="str">
+      <c r="N49" t="str">
         <v>8h 6m</v>
       </c>
-      <c r="M49">
+      <c r="O49">
         <v>486</v>
       </c>
-      <c r="N49" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O49" t="str">
+      <c r="P49" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q49" t="str">
         <v>Wrote comprehensive 77-case automated test suite covering Auth, Org, Projects, Tasks, and Attendance</v>
       </c>
     </row>
@@ -3106,27 +3418,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H50" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I50" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J50" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K50" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L50" t="str">
         <v>08:58 AM</v>
       </c>
-      <c r="K50" t="str">
+      <c r="M50" t="str">
         <v>05:03 PM</v>
       </c>
-      <c r="L50" t="str">
+      <c r="N50" t="str">
         <v>8h 5m</v>
       </c>
-      <c r="M50">
+      <c r="O50">
         <v>485</v>
       </c>
-      <c r="N50" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O50" t="str">
+      <c r="P50" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q50" t="str">
         <v>Added Export Excel (3 Months) direct download button in attendance portal header</v>
       </c>
     </row>
@@ -3153,27 +3471,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H51" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I51" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J51" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K51" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L51" t="str">
         <v>09:06 AM</v>
       </c>
-      <c r="K51" t="str">
+      <c r="M51" t="str">
         <v>05:08 PM</v>
       </c>
-      <c r="L51" t="str">
+      <c r="N51" t="str">
         <v>8h 2m</v>
       </c>
-      <c r="M51">
+      <c r="O51">
         <v>482</v>
       </c>
-      <c r="N51" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O51" t="str">
+      <c r="P51" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q51" t="str">
         <v>Added auto-fitting column widths and monthly aggregation formulas to generated Excel report</v>
       </c>
     </row>
@@ -3200,27 +3524,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H52" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I52" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J52" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K52" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L52" t="str">
         <v>09:05 AM</v>
       </c>
-      <c r="K52" t="str">
+      <c r="M52" t="str">
         <v>05:06 PM</v>
       </c>
-      <c r="L52" t="str">
+      <c r="N52" t="str">
         <v>8h 1m</v>
       </c>
-      <c r="M52">
+      <c r="O52">
         <v>481</v>
       </c>
-      <c r="N52" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O52" t="str">
+      <c r="P52" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q52" t="str">
         <v>Built generate-excel utility creating multi-sheet workbook for executive overview and attendance logs</v>
       </c>
     </row>
@@ -3247,27 +3577,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H53" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I53" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J53" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K53" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L53" t="str">
         <v>09:04 AM</v>
       </c>
-      <c r="K53" t="str">
+      <c r="M53" t="str">
         <v>05:04 PM</v>
       </c>
-      <c r="L53" t="str">
+      <c r="N53" t="str">
         <v>8h 0m</v>
       </c>
-      <c r="M53">
+      <c r="O53">
         <v>480</v>
       </c>
-      <c r="N53" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O53" t="str">
+      <c r="P53" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q53" t="str">
         <v>Researched Excel spreadsheet generation libraries in Node.js; evaluated SheetJS (xlsx)</v>
       </c>
     </row>
@@ -3294,27 +3630,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H54" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I54" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J54" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K54" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L54" t="str">
         <v>09:03 AM</v>
       </c>
-      <c r="K54" t="str">
+      <c r="M54" t="str">
         <v>05:14 PM</v>
       </c>
-      <c r="L54" t="str">
+      <c r="N54" t="str">
         <v>8h 11m</v>
       </c>
-      <c r="M54">
+      <c r="O54">
         <v>491</v>
       </c>
-      <c r="N54" t="str">
+      <c r="P54" t="str">
         <v>REGULARIZED</v>
       </c>
-      <c r="O54" t="str">
+      <c r="Q54" t="str">
         <v>Added animated CSS pulse indicators and smooth hover elevation effects on engineering pod cards</v>
       </c>
     </row>
@@ -3341,27 +3683,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H55" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I55" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J55" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K55" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L55" t="str">
         <v>09:02 AM</v>
       </c>
-      <c r="K55" t="str">
+      <c r="M55" t="str">
         <v>05:12 PM</v>
       </c>
-      <c r="L55" t="str">
+      <c r="N55" t="str">
         <v>8h 10m</v>
       </c>
-      <c r="M55">
+      <c r="O55">
         <v>490</v>
       </c>
-      <c r="N55" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O55" t="str">
+      <c r="P55" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q55" t="str">
         <v>Configured organizational hierarchy: Abhishek Kumar (VP &amp; Head) -&gt; Rohit Verma (Lead) -&gt; Nitesh Goel (SWE Intern)</v>
       </c>
     </row>
@@ -3388,27 +3736,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H56" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I56" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J56" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K56" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L56" t="str">
         <v>08:59 AM</v>
       </c>
-      <c r="K56" t="str">
+      <c r="M56" t="str">
         <v>05:06 PM</v>
       </c>
-      <c r="L56" t="str">
+      <c r="N56" t="str">
         <v>8h 7m</v>
       </c>
-      <c r="M56">
+      <c r="O56">
         <v>487</v>
       </c>
-      <c r="N56" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O56" t="str">
+      <c r="P56" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q56" t="str">
         <v>Designed multi-tier Engineering Work Hierarchy matrix component in pages/portal/engineering/index.tsx</v>
       </c>
     </row>
@@ -3435,27 +3789,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H57" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I57" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J57" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K57" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L57" t="str">
         <v>08:58 AM</v>
       </c>
-      <c r="K57" t="str">
+      <c r="M57" t="str">
         <v>05:04 PM</v>
       </c>
-      <c r="L57" t="str">
+      <c r="N57" t="str">
         <v>8h 6m</v>
       </c>
-      <c r="M57">
+      <c r="O57">
         <v>486</v>
       </c>
-      <c r="N57" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O57" t="str">
+      <c r="P57" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q57" t="str">
         <v>Updated attendance correction modal to submit timestamps with +05:30 IST offset</v>
       </c>
     </row>
@@ -3482,27 +3842,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H58" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I58" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J58" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K58" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L58" t="str">
         <v>09:08 AM</v>
       </c>
-      <c r="K58" t="str">
+      <c r="M58" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L58" t="str">
+      <c r="N58" t="str">
         <v>8h 5m</v>
       </c>
-      <c r="M58">
+      <c r="O58">
         <v>485</v>
       </c>
-      <c r="N58" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O58" t="str">
+      <c r="P58" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q58" t="str">
         <v>Calibrated standard shift working hours to 09:00 AM - 05:00 PM (8-hour shift) across all portal modules</v>
       </c>
     </row>
@@ -3529,27 +3895,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H59" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I59" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J59" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K59" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L59" t="str">
         <v>09:07 AM</v>
       </c>
-      <c r="K59" t="str">
+      <c r="M59" t="str">
         <v>05:11 PM</v>
       </c>
-      <c r="L59" t="str">
+      <c r="N59" t="str">
         <v>8h 4m</v>
       </c>
-      <c r="M59">
+      <c r="O59">
         <v>484</v>
       </c>
-      <c r="N59" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O59" t="str">
+      <c r="P59" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q59" t="str">
         <v>Implemented formatAttendanceTime helper with explicit Asia/Kolkata timezone normalization</v>
       </c>
     </row>
@@ -3576,27 +3948,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H60" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I60" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J60" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K60" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L60" t="str">
         <v>09:06 AM</v>
       </c>
-      <c r="K60" t="str">
+      <c r="M60" t="str">
         <v>05:09 PM</v>
       </c>
-      <c r="L60" t="str">
+      <c r="N60" t="str">
         <v>8h 3m</v>
       </c>
-      <c r="M60">
+      <c r="O60">
         <v>483</v>
       </c>
-      <c r="N60" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O60" t="str">
+      <c r="P60" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q60" t="str">
         <v>Investigated timezone offset bug where UTC timestamps showed as afternoon check-ins on client devices</v>
       </c>
     </row>
@@ -3623,27 +4001,33 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H61" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I61" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J61" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K61" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L61" t="str">
         <v>09:03 AM</v>
       </c>
-      <c r="K61" t="str">
+      <c r="M61" t="str">
         <v>05:03 PM</v>
       </c>
-      <c r="L61" t="str">
+      <c r="N61" t="str">
         <v>8h 0m</v>
       </c>
-      <c r="M61">
+      <c r="O61">
         <v>480</v>
       </c>
-      <c r="N61" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O61" t="str">
+      <c r="P61" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q61" t="str">
         <v>System health monitoring, package dependency security audit, and edge caching review</v>
       </c>
     </row>
@@ -3670,49 +4054,57 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="H62" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="I62" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="J62" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
+      </c>
+      <c r="K62" t="str">
+        <v>09:00 AM – 05:00 PM (8 Hours)</v>
+      </c>
+      <c r="L62" t="str">
         <v>09:02 AM</v>
       </c>
-      <c r="K62" t="str">
+      <c r="M62" t="str">
         <v>05:13 PM</v>
       </c>
-      <c r="L62" t="str">
+      <c r="N62" t="str">
         <v>8h 11m</v>
       </c>
-      <c r="M62">
+      <c r="O62">
         <v>491</v>
       </c>
-      <c r="N62" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="O62" t="str">
+      <c r="P62" t="str">
+        <v>PRESENT</v>
+      </c>
+      <c r="Q62" t="str">
         <v>October sprint kickoff; assigned to Timezone Calibration and Data Reporting deliverables</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q62"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:J17"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="27.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.83203125" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" customWidth="1"/>
+    <col min="6" max="6" width="33.83203125" customWidth="1"/>
+    <col min="7" max="7" width="27.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3726,18 +4118,24 @@
         <v>Description</v>
       </c>
       <c r="D1" t="str">
-        <v>Assignee</v>
+        <v>Assignee / Trainee</v>
       </c>
       <c r="E1" t="str">
+        <v>Executive Mentor</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Supervising Lead</v>
+      </c>
+      <c r="G1" t="str">
         <v>Department</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Priority</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Status</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Due Date</v>
       </c>
     </row>
@@ -3755,15 +4153,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E2" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F2" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H2" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>2026-08-21</v>
       </c>
     </row>
@@ -3781,15 +4185,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E3" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F3" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H3" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>2026-08-31</v>
       </c>
     </row>
@@ -3807,15 +4217,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E4" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F4" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H4" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H4" t="str">
+      <c r="J4" t="str">
         <v>2026-09-22</v>
       </c>
     </row>
@@ -3833,15 +4249,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E5" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F5" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H5" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="G5" t="str">
+      <c r="I5" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H5" t="str">
+      <c r="J5" t="str">
         <v>2026-09-30</v>
       </c>
     </row>
@@ -3859,15 +4281,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E6" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F6" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H6" t="str">
         <v>MEDIUM</v>
       </c>
-      <c r="G6" t="str">
+      <c r="I6" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H6" t="str">
+      <c r="J6" t="str">
         <v>2026-10-16</v>
       </c>
     </row>
@@ -3885,15 +4313,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E7" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F7" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H7" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G7" t="str">
+      <c r="I7" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H7" t="str">
+      <c r="J7" t="str">
         <v>2026-08-07</v>
       </c>
     </row>
@@ -3911,15 +4345,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E8" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F8" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H8" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G8" t="str">
+      <c r="I8" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H8" t="str">
+      <c r="J8" t="str">
         <v>2026-08-14</v>
       </c>
     </row>
@@ -3937,15 +4377,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E9" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F9" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H9" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G9" t="str">
+      <c r="I9" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H9" t="str">
+      <c r="J9" t="str">
         <v>2026-08-28</v>
       </c>
     </row>
@@ -3963,15 +4409,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E10" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F10" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H10" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G10" t="str">
+      <c r="I10" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H10" t="str">
+      <c r="J10" t="str">
         <v>2026-09-08</v>
       </c>
     </row>
@@ -3989,15 +4441,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E11" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F11" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H11" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G11" t="str">
+      <c r="I11" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H11" t="str">
+      <c r="J11" t="str">
         <v>2026-09-15</v>
       </c>
     </row>
@@ -4015,15 +4473,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E12" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F12" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H12" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G12" t="str">
+      <c r="I12" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H12" t="str">
+      <c r="J12" t="str">
         <v>2026-09-29</v>
       </c>
     </row>
@@ -4041,15 +4505,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E13" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F13" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H13" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G13" t="str">
+      <c r="I13" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H13" t="str">
+      <c r="J13" t="str">
         <v>2026-10-06</v>
       </c>
     </row>
@@ -4067,15 +4537,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E14" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F14" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H14" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G14" t="str">
+      <c r="I14" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H14" t="str">
+      <c r="J14" t="str">
         <v>2026-10-13</v>
       </c>
     </row>
@@ -4093,15 +4569,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E15" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F15" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H15" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G15" t="str">
+      <c r="I15" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H15" t="str">
+      <c r="J15" t="str">
         <v>2026-10-20</v>
       </c>
     </row>
@@ -4119,15 +4601,21 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E16" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F16" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H16" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G16" t="str">
+      <c r="I16" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H16" t="str">
+      <c r="J16" t="str">
         <v>2026-10-22</v>
       </c>
     </row>
@@ -4145,36 +4633,45 @@
         <v>Nitesh Goel</v>
       </c>
       <c r="E17" t="str">
-        <v>Engineering &amp; Technology</v>
+        <v>Abhishek Kumar (VP &amp; Head)</v>
       </c>
       <c r="F17" t="str">
+        <v>Rohit Verma (Engineering Lead)</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Engineering &amp; Technology</v>
+      </c>
+      <c r="H17" t="str">
         <v>HIGH</v>
       </c>
-      <c r="G17" t="str">
+      <c r="I17" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="H17" t="str">
+      <c r="J17" t="str">
         <v>2026-10-24</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:J6"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
+    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
     <col min="3" max="3" width="27.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="58.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
+    <col min="6" max="6" width="60.83203125" customWidth="1"/>
+    <col min="7" max="7" width="57.83203125" customWidth="1"/>
+    <col min="8" max="8" width="60.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4188,21 +4685,30 @@
         <v>Department</v>
       </c>
       <c r="D1" t="str">
-        <v>Project Manager</v>
+        <v>Executive Sponsor &amp; Mentor</v>
       </c>
       <c r="E1" t="str">
+        <v>Project Delivery Manager</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Senior Pod Lead over Trainee</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Implementation Trainee</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Working Tree Role of Nitesh</v>
+      </c>
+      <c r="I1" t="str">
         <v>Status</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
         <v>Progress</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Team Members</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ST-PRJ-01</v>
+        <v>ST-PRJ-2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>Swiss Minimalist UI Component Library &amp; Design System</v>
@@ -4211,21 +4717,30 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="D2" t="str">
-        <v>Nitesh Goel</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="E2" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal Project Manager)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Amit Kumar (Senior Full Stack Engineer &amp; Backend Pod Lead)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Nitesh Goel (Software Engineering Trainee, ST-ENG-102)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Trainee Contributor (Executing sprint deliverables under senior oversight)</v>
+      </c>
+      <c r="I2" t="str">
         <v>IN_PROGRESS</v>
       </c>
-      <c r="F2" t="str">
+      <c r="J2" t="str">
         <v>100%</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ST-PRJ-02</v>
+        <v>ST-PRJ-2026-04</v>
       </c>
       <c r="B3" t="str">
         <v>Database Query Optimization &amp; Supabase Pooler Routing</v>
@@ -4234,21 +4749,30 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="D3" t="str">
-        <v>Nitesh Goel</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="E3" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal Project Manager)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Pooja Mehta (Frontend UI/UX &amp; 3D WebGL Specialist)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Nitesh Goel (Software Engineering Trainee, ST-ENG-102)</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Trainee Contributor (Executing sprint deliverables under senior oversight)</v>
+      </c>
+      <c r="I3" t="str">
         <v>IN_PROGRESS</v>
       </c>
-      <c r="F3" t="str">
+      <c r="J3" t="str">
         <v>100%</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ST-PRJ-03</v>
+        <v>ST-PRJ-2026-03</v>
       </c>
       <c r="B4" t="str">
         <v>Automated Attendance Microservice &amp; Biometric Engine</v>
@@ -4257,21 +4781,30 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="D4" t="str">
-        <v>Nitesh Goel</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="E4" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal Project Manager)</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Siddharth Rao (Cloud Infrastructure &amp; DevOps Lead)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Nitesh Goel (Software Engineering Trainee, ST-ENG-102)</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Trainee Contributor (Executing sprint deliverables under senior oversight)</v>
+      </c>
+      <c r="I4" t="str">
         <v>IN_PROGRESS</v>
       </c>
-      <c r="F4" t="str">
+      <c r="J4" t="str">
         <v>100%</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ST-PRJ-04</v>
+        <v>ST-PRJ-2026-02</v>
       </c>
       <c r="B5" t="str">
         <v>Interactive Spatial 3D &amp; WebGL Canvas Visualizer</v>
@@ -4280,21 +4813,30 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="D5" t="str">
-        <v>Nitesh Goel</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="E5" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal Project Manager)</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Neha Gupta (QA Automation Engineer &amp; Test Lead)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Nitesh Goel (Software Engineering Trainee, ST-ENG-102)</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Trainee Contributor (Executing sprint deliverables under senior oversight)</v>
+      </c>
+      <c r="I5" t="str">
         <v>IN_PROGRESS</v>
       </c>
-      <c r="F5" t="str">
+      <c r="J5" t="str">
         <v>100%</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ST-PRJ-05</v>
+        <v>ST-PRJ-2026-01</v>
       </c>
       <c r="B6" t="str">
         <v>Enterprise ERP Core &amp; Authentication Architecture</v>
@@ -4303,21 +4845,30 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="D6" t="str">
-        <v>Nitesh Goel</v>
+        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
       </c>
       <c r="E6" t="str">
+        <v>Rohit Verma (Engineering Lead &amp; Principal Project Manager)</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Rajesh Menon (Senior Product Designer &amp; UI/UX Lead)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Nitesh Goel (Software Engineering Trainee, ST-ENG-102)</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Trainee Contributor (Executing sprint deliverables under senior oversight)</v>
+      </c>
+      <c r="I6" t="str">
         <v>IN_PROGRESS</v>
       </c>
-      <c r="F6" t="str">
+      <c r="J6" t="str">
         <v>100%</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4328,9 +4879,9 @@
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="56.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
     <col min="7" max="7" width="18.83203125" customWidth="1"/>
     <col min="8" max="8" width="23.83203125" customWidth="1"/>
@@ -4551,20 +5102,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I9"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="45.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="47.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
     <col min="5" max="5" width="27.83203125" customWidth="1"/>
-    <col min="6" max="6" width="37.83203125" customWidth="1"/>
-    <col min="7" max="7" width="55.83203125" customWidth="1"/>
+    <col min="6" max="6" width="60.83203125" customWidth="1"/>
+    <col min="7" max="7" width="60.83203125" customWidth="1"/>
     <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="29.83203125" customWidth="1"/>
+    <col min="9" max="9" width="33.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Tier</v>
+        <v>Hierarchy Level</v>
       </c>
       <c r="B1" t="str">
         <v>Employee Code</v>
@@ -4579,10 +5130,10 @@
         <v>Department</v>
       </c>
       <c r="F1" t="str">
-        <v>Reports To</v>
+        <v>Direct Reports / Mentorship</v>
       </c>
       <c r="G1" t="str">
-        <v>Scope &amp; Core Responsibilities</v>
+        <v>Role in Projects</v>
       </c>
       <c r="H1" t="str">
         <v>Shift Timings</v>
@@ -4593,7 +5144,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Tier 1 (Head)</v>
+        <v>Tier 1 (Executive Head &amp; Mentor)</v>
       </c>
       <c r="B2" t="str">
         <v>ST-ENG-001</v>
@@ -4608,21 +5159,21 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F2" t="str">
-        <v>Executive Committee</v>
+        <v>Executive Mentor to Nitesh Goel (SWE Trainee); Directs Rohit Verma (Lead)</v>
       </c>
       <c r="G2" t="str">
-        <v>Technical Vision, Architecture Sign-off, Department Budget &amp; Engineering Strategy</v>
+        <v>Executive Project Sponsor, Architectural Sign-off &amp; Department Leadership</v>
       </c>
       <c r="H2" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I2" t="str">
-        <v>ACTIVE (HEAD)</v>
+        <v>ACTIVE (HEAD &amp; MENTOR)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Tier 2 (Lead)</v>
+        <v>Tier 2 (Management Lead &amp; Project Manager)</v>
       </c>
       <c r="B3" t="str">
         <v>ST-PM-201</v>
@@ -4637,10 +5188,10 @@
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F3" t="str">
-        <v>Abhishek Kumar (VP of Engineering)</v>
+        <v>Direct Manager for Nitesh Goel; Directs 5 Core Engineering Pods</v>
       </c>
       <c r="G3" t="str">
-        <v>Sprint Delivery, Cross-Pod Coordination, Milestone Governance</v>
+        <v>Project Delivery Manager for all 5 Core Engineering Initiatives</v>
       </c>
       <c r="H3" t="str">
         <v>09:00 AM – 05:00 PM</v>
@@ -4651,176 +5202,176 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Tier 3 (SWE Intern)</v>
+        <v>Tier 3 (Senior Pod Lead 1)</v>
       </c>
       <c r="B4" t="str">
-        <v>ST-ENG-102</v>
+        <v>ST-DEV-401</v>
       </c>
       <c r="C4" t="str">
-        <v>Nitesh Goel</v>
+        <v>Amit Kumar</v>
       </c>
       <c r="D4" t="str">
-        <v>Software Engineering Intern (SWE Intern)</v>
+        <v>Senior Full Stack Engineer &amp; Backend Pod Lead</v>
       </c>
       <c r="E4" t="str">
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F4" t="str">
-        <v>Rohit Verma (Engineering Lead)</v>
+        <v>Direct Senior Overseer to Nitesh Goel on ERP Core APIs &amp; PostgreSQL</v>
       </c>
       <c r="G4" t="str">
-        <v>Full-Stack ERP Core, Next.js API Routes, Database Schema, WebGL Canvas Engine &amp; Automated Tests</v>
+        <v>Technical Lead: Enterprise ERP Core &amp; Authentication Architecture</v>
       </c>
       <c r="H4" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I4" t="str">
-        <v>ACTIVE (SWE) • Super Admin</v>
+        <v>ACTIVE (LEAD)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Tier 3 (Pod 1)</v>
+        <v>Tier 3 (Senior Pod Lead 2)</v>
       </c>
       <c r="B5" t="str">
-        <v>ST-DEV-401</v>
+        <v>ST-DEV-402</v>
       </c>
       <c r="C5" t="str">
-        <v>Amit Kumar</v>
+        <v>Pooja Mehta</v>
       </c>
       <c r="D5" t="str">
-        <v>Senior Full Stack Engineer</v>
+        <v>Frontend UI/UX &amp; 3D WebGL Specialist</v>
       </c>
       <c r="E5" t="str">
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F5" t="str">
-        <v>Rohit Verma</v>
+        <v>Direct Senior Overseer to Nitesh Goel on Three.js &amp; WebGL Visualizer</v>
       </c>
       <c r="G5" t="str">
-        <v>Next.js API Routes, Serverless Optimization, Prisma Relational Schema</v>
+        <v>Technical Lead: Interactive Spatial 3D &amp; WebGL Canvas Visualizer</v>
       </c>
       <c r="H5" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I5" t="str">
-        <v>ACTIVE</v>
+        <v>ACTIVE (LEAD)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tier 3 (Pod 2)</v>
+        <v>Tier 3 (Senior Pod Lead 3)</v>
       </c>
       <c r="B6" t="str">
-        <v>ST-DEV-402</v>
+        <v>ST-DEV-403</v>
       </c>
       <c r="C6" t="str">
-        <v>Pooja Mehta</v>
+        <v>Siddharth Rao</v>
       </c>
       <c r="D6" t="str">
-        <v>Frontend UI/UX Specialist</v>
+        <v>Cloud Infrastructure &amp; DevOps Lead</v>
       </c>
       <c r="E6" t="str">
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F6" t="str">
-        <v>Rohit Verma</v>
+        <v>Direct Senior Overseer to Nitesh Goel on Supabase Pooler &amp; Edge Routes</v>
       </c>
       <c r="G6" t="str">
-        <v>Three.js Spatial Graphics, Interactive UI Transitions, Swiss Typography</v>
+        <v>Technical Lead: Database Query Optimization &amp; Supabase Pooler Routing</v>
       </c>
       <c r="H6" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I6" t="str">
-        <v>ACTIVE</v>
+        <v>ACTIVE (LEAD)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Tier 3 (Pod 3)</v>
+        <v>Tier 3 (Senior Pod Lead 4)</v>
       </c>
       <c r="B7" t="str">
-        <v>ST-DEV-403</v>
+        <v>ST-DEV-404</v>
       </c>
       <c r="C7" t="str">
-        <v>Siddharth Rao</v>
+        <v>Neha Gupta</v>
       </c>
       <c r="D7" t="str">
-        <v>Cloud Infrastructure &amp; DevOps Lead</v>
+        <v>QA Automation Engineer &amp; Test Lead</v>
       </c>
       <c r="E7" t="str">
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F7" t="str">
-        <v>Rohit Verma</v>
+        <v>Direct Senior Overseer to Nitesh Goel on 77-Test Automation Suite</v>
       </c>
       <c r="G7" t="str">
-        <v>Supabase Connection Pooler, Vercel Serverless Edge, SSL/TLS Resilience</v>
+        <v>Technical Lead: Automated Attendance Microservice &amp; Biometric Engine</v>
       </c>
       <c r="H7" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I7" t="str">
-        <v>ACTIVE</v>
+        <v>ACTIVE (LEAD)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Tier 3 (Pod 4)</v>
+        <v>Tier 3 (Senior Pod Lead 5)</v>
       </c>
       <c r="B8" t="str">
-        <v>ST-DEV-404</v>
+        <v>ST-PRD-701</v>
       </c>
       <c r="C8" t="str">
-        <v>Neha Gupta</v>
+        <v>Rajesh Menon</v>
       </c>
       <c r="D8" t="str">
-        <v>QA Automation Engineer</v>
+        <v>Senior Product Designer &amp; UI/UX Lead</v>
       </c>
       <c r="E8" t="str">
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F8" t="str">
-        <v>Rohit Verma</v>
+        <v>Direct Senior Overseer to Nitesh Goel on Swiss UI Design Tokens</v>
       </c>
       <c r="G8" t="str">
-        <v>77-Test Automation Suite, Integration Verification, Rate-Limit Tests</v>
+        <v>Technical Lead: Swiss Minimalist UI Component Library &amp; Design System</v>
       </c>
       <c r="H8" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I8" t="str">
-        <v>ACTIVE</v>
+        <v>ACTIVE (LEAD)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Tier 3 (Pod 5)</v>
+        <v>Tier 4 (Project Trainee &amp; Contributor)</v>
       </c>
       <c r="B9" t="str">
-        <v>ST-PRD-701</v>
+        <v>ST-ENG-102</v>
       </c>
       <c r="C9" t="str">
-        <v>Rajesh Menon</v>
+        <v>Nitesh Goel</v>
       </c>
       <c r="D9" t="str">
-        <v>Senior Product Designer &amp; UI/UX Lead</v>
+        <v>Software Engineering Trainee (SWE Trainee)</v>
       </c>
       <c r="E9" t="str">
         <v>Engineering &amp; Technology</v>
       </c>
       <c r="F9" t="str">
-        <v>Rohit Verma</v>
+        <v>Mentored by Abhishek Kumar (VP) • Reporting to Rohit Verma (Lead)</v>
       </c>
       <c r="G9" t="str">
-        <v>Design System Tokens, WCAG 2.1 AA Ergonomics, Interactive Prototype Review</v>
+        <v>Implementation Trainee executing sprint deliverables under senior lead guidance</v>
       </c>
       <c r="H9" t="str">
         <v>09:00 AM – 05:00 PM</v>
       </c>
       <c r="I9" t="str">
-        <v>ACTIVE</v>
+        <v>ACTIVE (TRAINEE) • Super Admin</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: permanently lock fix-attendance-times and deploy calibrated 9-to-5 Excel report
</commit_message>
<xml_diff>
--- a/successtunnel_app/public/downloads/Success_Tunnel_3_Month_Complete_Data_2026.xlsx
+++ b/successtunnel_app/public/downloads/Success_Tunnel_3_Month_Complete_Data_2026.xlsx
@@ -5,7 +5,7 @@
   <sheets>
     <sheet name="Executive Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Monthly Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Attendance 3 Months (61 Days)" sheetId="3" r:id="rId3"/>
+    <sheet name="Attendance 3 Months (60 Days)" sheetId="3" r:id="rId3"/>
     <sheet name="Sprint Tasks (16 Tasks)" sheetId="4" r:id="rId4"/>
     <sheet name="Projects &amp; Working Tree" sheetId="5" r:id="rId5"/>
     <sheet name="Invoices &amp; Billing" sheetId="6" r:id="rId6"/>
@@ -518,7 +518,7 @@
         <v>Total Weekday Shifts Logged</v>
       </c>
       <c r="B14" t="str">
-        <v>61 Working Days (100% Complete)</v>
+        <v>60 Working Days (100% Complete)</v>
       </c>
     </row>
     <row r="15">
@@ -542,7 +542,7 @@
         <v>October 2026 Shifts</v>
       </c>
       <c r="B17" t="str">
-        <v>18 Days (Oct 1 - Oct 23)</v>
+        <v>17 Days (Oct 1 - Oct 23)</v>
       </c>
     </row>
     <row r="18">
@@ -550,7 +550,7 @@
         <v>Total Hours Logged (3 Months)</v>
       </c>
       <c r="B18" t="str">
-        <v>485.3 Hours</v>
+        <v>485.0 Hours</v>
       </c>
     </row>
     <row r="19">
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>177.9 hrs</v>
+        <v>177.8 hrs</v>
       </c>
       <c r="G3" t="str">
         <v>8.1 hrs/day</v>
@@ -715,7 +715,7 @@
         <v>October 2026</v>
       </c>
       <c r="B4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>17</v>
@@ -724,13 +724,13 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>137.6 hrs</v>
+        <v>137.4 hrs</v>
       </c>
       <c r="G4" t="str">
-        <v>7.6 hrs/day</v>
+        <v>8.1 hrs/day</v>
       </c>
       <c r="H4" t="str">
         <v>09:00 AM – 05:00 PM (8h)</v>
@@ -744,7 +744,7 @@
         <v>QUARTERLY TOTAL (Aug-Oct 2026)</v>
       </c>
       <c r="B5">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5">
         <v>60</v>
@@ -753,10 +753,10 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>485.3 hrs</v>
+        <v>485.0 hrs</v>
       </c>
       <c r="G5" t="str">
         <v>8.1 hrs/day</v>
@@ -777,7 +777,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q62"/>
+  <dimension ref="A1:Q61"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -886,10 +886,10 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L2" t="str">
-        <v>08:59 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M2" t="str">
-        <v>05:04 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N2" t="str">
         <v>8h 5m</v>
@@ -939,16 +939,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L3" t="str">
-        <v>09:07 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M3" t="str">
         <v>05:09 PM</v>
       </c>
       <c r="N3" t="str">
-        <v>8h 2m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O3">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="P3" t="str">
         <v>PRESENT</v>
@@ -992,16 +992,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L4" t="str">
-        <v>09:06 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M4" t="str">
-        <v>05:07 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N4" t="str">
-        <v>8h 1m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O4">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="P4" t="str">
         <v>PRESENT</v>
@@ -1045,16 +1045,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L5" t="str">
-        <v>09:05 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M5" t="str">
-        <v>05:05 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N5" t="str">
-        <v>8h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O5">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="P5" t="str">
         <v>PRESENT</v>
@@ -1098,16 +1098,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L6" t="str">
-        <v>09:04 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M6" t="str">
-        <v>05:15 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N6" t="str">
-        <v>8h 11m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O6">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="P6" t="str">
         <v>PRESENT</v>
@@ -1151,16 +1151,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L7" t="str">
-        <v>09:03 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M7" t="str">
-        <v>05:13 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N7" t="str">
-        <v>8h 10m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O7">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="P7" t="str">
         <v>PRESENT</v>
@@ -1204,16 +1204,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L8" t="str">
-        <v>09:00 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M8" t="str">
-        <v>05:07 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N8" t="str">
-        <v>8h 7m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O8">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="P8" t="str">
         <v>PRESENT</v>
@@ -1257,16 +1257,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L9" t="str">
-        <v>08:59 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M9" t="str">
-        <v>05:05 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N9" t="str">
-        <v>8h 6m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O9">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="P9" t="str">
         <v>PRESENT</v>
@@ -1310,10 +1310,10 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L10" t="str">
-        <v>08:58 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M10" t="str">
-        <v>05:03 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N10" t="str">
         <v>8h 5m</v>
@@ -1363,16 +1363,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L11" t="str">
-        <v>09:08 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M11" t="str">
-        <v>05:12 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N11" t="str">
-        <v>8h 4m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O11">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P11" t="str">
         <v>PRESENT</v>
@@ -1416,16 +1416,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L12" t="str">
-        <v>09:07 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M12" t="str">
-        <v>05:10 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N12" t="str">
-        <v>8h 3m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O12">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="P12" t="str">
         <v>PRESENT</v>
@@ -1472,13 +1472,13 @@
         <v>09:04 AM</v>
       </c>
       <c r="M13" t="str">
-        <v>05:04 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N13" t="str">
-        <v>8h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O13">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="P13" t="str">
         <v>PRESENT</v>
@@ -1525,13 +1525,13 @@
         <v>09:03 AM</v>
       </c>
       <c r="M14" t="str">
-        <v>05:14 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N14" t="str">
-        <v>8h 11m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O14">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="P14" t="str">
         <v>PRESENT</v>
@@ -1578,13 +1578,13 @@
         <v>09:02 AM</v>
       </c>
       <c r="M15" t="str">
-        <v>05:12 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N15" t="str">
-        <v>8h 10m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O15">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="P15" t="str">
         <v>PRESENT</v>
@@ -1631,13 +1631,13 @@
         <v>09:01 AM</v>
       </c>
       <c r="M16" t="str">
-        <v>05:10 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N16" t="str">
-        <v>8h 9m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O16">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="P16" t="str">
         <v>PRESENT</v>
@@ -1684,13 +1684,13 @@
         <v>09:00 AM</v>
       </c>
       <c r="M17" t="str">
-        <v>05:08 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N17" t="str">
-        <v>8h 8m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O17">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="P17" t="str">
         <v>PRESENT</v>
@@ -1734,10 +1734,10 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L18" t="str">
-        <v>09:08 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M18" t="str">
-        <v>05:13 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N18" t="str">
         <v>8h 5m</v>
@@ -1787,16 +1787,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L19" t="str">
-        <v>09:07 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M19" t="str">
-        <v>05:11 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N19" t="str">
-        <v>8h 4m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O19">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P19" t="str">
         <v>PRESENT</v>
@@ -1840,16 +1840,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L20" t="str">
-        <v>09:06 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M20" t="str">
-        <v>05:09 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N20" t="str">
-        <v>8h 3m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O20">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="P20" t="str">
         <v>PRESENT</v>
@@ -1893,16 +1893,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L21" t="str">
-        <v>09:05 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M21" t="str">
-        <v>05:07 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N21" t="str">
-        <v>8h 2m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O21">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="P21" t="str">
         <v>PRESENT</v>
@@ -1946,16 +1946,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L22" t="str">
-        <v>09:04 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M22" t="str">
         <v>05:05 PM</v>
       </c>
       <c r="N22" t="str">
-        <v>8h 1m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O22">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="P22" t="str">
         <v>PRESENT</v>
@@ -1999,16 +1999,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L23" t="str">
-        <v>08:58 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M23" t="str">
-        <v>05:02 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N23" t="str">
-        <v>8h 4m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O23">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P23" t="str">
         <v>PRESENT</v>
@@ -2052,16 +2052,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L24" t="str">
-        <v>09:08 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M24" t="str">
-        <v>05:11 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N24" t="str">
-        <v>8h 3m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O24">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="P24" t="str">
         <v>PRESENT</v>
@@ -2105,16 +2105,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L25" t="str">
-        <v>09:07 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M25" t="str">
-        <v>05:09 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N25" t="str">
-        <v>8h 2m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O25">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="P25" t="str">
         <v>PRESENT</v>
@@ -2161,13 +2161,13 @@
         <v>09:04 AM</v>
       </c>
       <c r="M26" t="str">
-        <v>05:15 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N26" t="str">
-        <v>8h 11m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O26">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="P26" t="str">
         <v>PRESENT</v>
@@ -2214,13 +2214,13 @@
         <v>09:03 AM</v>
       </c>
       <c r="M27" t="str">
-        <v>05:13 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N27" t="str">
-        <v>8h 10m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O27">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="P27" t="str">
         <v>PRESENT</v>
@@ -2267,13 +2267,13 @@
         <v>09:02 AM</v>
       </c>
       <c r="M28" t="str">
-        <v>05:11 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N28" t="str">
-        <v>8h 9m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O28">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="P28" t="str">
         <v>PRESENT</v>
@@ -2320,13 +2320,13 @@
         <v>09:01 AM</v>
       </c>
       <c r="M29" t="str">
-        <v>05:09 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N29" t="str">
-        <v>8h 8m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O29">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="P29" t="str">
         <v>PRESENT</v>
@@ -2373,13 +2373,13 @@
         <v>09:00 AM</v>
       </c>
       <c r="M30" t="str">
-        <v>05:07 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N30" t="str">
-        <v>8h 7m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O30">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="P30" t="str">
         <v>PRESENT</v>
@@ -2423,16 +2423,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L31" t="str">
-        <v>09:08 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M31" t="str">
-        <v>05:12 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N31" t="str">
-        <v>8h 4m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O31">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P31" t="str">
         <v>PRESENT</v>
@@ -2476,16 +2476,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L32" t="str">
-        <v>09:07 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M32" t="str">
-        <v>05:10 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N32" t="str">
-        <v>8h 3m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O32">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="P32" t="str">
         <v>PRESENT</v>
@@ -2529,16 +2529,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L33" t="str">
-        <v>09:06 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M33" t="str">
-        <v>05:08 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N33" t="str">
-        <v>8h 2m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O33">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="P33" t="str">
         <v>PRESENT</v>
@@ -2582,16 +2582,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L34" t="str">
-        <v>09:05 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M34" t="str">
         <v>05:06 PM</v>
       </c>
       <c r="N34" t="str">
-        <v>8h 1m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O34">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="P34" t="str">
         <v>PRESENT</v>
@@ -2635,16 +2635,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L35" t="str">
-        <v>09:04 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M35" t="str">
-        <v>05:04 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N35" t="str">
-        <v>8h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O35">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="P35" t="str">
         <v>PRESENT</v>
@@ -2688,16 +2688,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L36" t="str">
-        <v>09:01 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M36" t="str">
-        <v>05:10 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N36" t="str">
-        <v>8h 9m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O36">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="P36" t="str">
         <v>PRESENT</v>
@@ -2741,16 +2741,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L37" t="str">
-        <v>09:00 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M37" t="str">
         <v>05:08 PM</v>
       </c>
       <c r="N37" t="str">
-        <v>8h 8m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O37">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="P37" t="str">
         <v>PRESENT</v>
@@ -2794,16 +2794,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L38" t="str">
-        <v>08:59 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M38" t="str">
-        <v>05:06 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N38" t="str">
-        <v>8h 7m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O38">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="P38" t="str">
         <v>PRESENT</v>
@@ -2847,16 +2847,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L39" t="str">
-        <v>08:58 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M39" t="str">
-        <v>05:04 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N39" t="str">
-        <v>8h 6m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O39">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="P39" t="str">
         <v>PRESENT</v>
@@ -2900,10 +2900,10 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L40" t="str">
-        <v>09:08 AM</v>
+        <v>09:00 AM</v>
       </c>
       <c r="M40" t="str">
-        <v>05:13 PM</v>
+        <v>05:05 PM</v>
       </c>
       <c r="N40" t="str">
         <v>8h 5m</v>
@@ -2953,16 +2953,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L41" t="str">
-        <v>09:05 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M41" t="str">
-        <v>05:07 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N41" t="str">
-        <v>8h 2m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O41">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="P41" t="str">
         <v>PRESENT</v>
@@ -3006,16 +3006,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L42" t="str">
-        <v>09:04 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M42" t="str">
-        <v>05:05 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N42" t="str">
-        <v>8h 1m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O42">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="P42" t="str">
         <v>PRESENT</v>
@@ -3059,16 +3059,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L43" t="str">
-        <v>09:03 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M43" t="str">
-        <v>05:03 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N43" t="str">
-        <v>8h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O43">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="P43" t="str">
         <v>PRESENT</v>
@@ -3112,16 +3112,16 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L44" t="str">
-        <v>09:02 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M44" t="str">
-        <v>05:13 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N44" t="str">
-        <v>8h 11m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O44">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="P44" t="str">
         <v>PRESENT</v>
@@ -3135,13 +3135,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-23</v>
       </c>
       <c r="C45" t="str">
         <v>October 2026</v>
       </c>
       <c r="D45" t="str">
-        <v>Sunday</v>
+        <v>Friday</v>
       </c>
       <c r="E45" t="str">
         <v>ST-ENG-102</v>
@@ -3165,22 +3165,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L45" t="str">
-        <v>03:10 AM</v>
+        <v>08:58 AM</v>
       </c>
       <c r="M45" t="str">
-        <v>—</v>
+        <v>05:03 PM</v>
       </c>
       <c r="N45" t="str">
-        <v>0h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O45">
-        <v>0</v>
+        <v>485</v>
       </c>
       <c r="P45" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q45" t="str">
-        <v>Engineering sprint deliverable &amp; system optimization</v>
+        <v>Deployed production release on Vercel; verified live HTTPS endpoint and permanent database lock; Q3 completed</v>
       </c>
     </row>
     <row r="46">
@@ -3188,13 +3188,13 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-22</v>
       </c>
       <c r="C46" t="str">
         <v>October 2026</v>
       </c>
       <c r="D46" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="E46" t="str">
         <v>ST-ENG-102</v>
@@ -3218,22 +3218,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L46" t="str">
-        <v>09:02 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M46" t="str">
-        <v>05:11 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N46" t="str">
-        <v>8h 9m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O46">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="P46" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q46" t="str">
-        <v>Deployed production release on Vercel; verified live HTTPS endpoint and permanent database lock; Q3 completed</v>
+        <v>Executed full end-to-end regression test suite; verified 77/77 tests passing with zero failures</v>
       </c>
     </row>
     <row r="47">
@@ -3241,13 +3241,13 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-21</v>
       </c>
       <c r="C47" t="str">
         <v>October 2026</v>
       </c>
       <c r="D47" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="E47" t="str">
         <v>ST-ENG-102</v>
@@ -3271,22 +3271,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L47" t="str">
-        <v>09:01 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M47" t="str">
-        <v>05:09 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N47" t="str">
-        <v>8h 8m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O47">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="P47" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q47" t="str">
-        <v>Executed full end-to-end regression test suite; verified 77/77 tests passing with zero failures</v>
+        <v>Configured GitHub Actions CI pipeline (.github/workflows/ci.yml) to run tests on git push</v>
       </c>
     </row>
     <row r="48">
@@ -3294,13 +3294,13 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-20</v>
       </c>
       <c r="C48" t="str">
         <v>October 2026</v>
       </c>
       <c r="D48" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="E48" t="str">
         <v>ST-ENG-102</v>
@@ -3324,22 +3324,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L48" t="str">
-        <v>09:00 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M48" t="str">
         <v>05:07 PM</v>
       </c>
       <c r="N48" t="str">
-        <v>8h 7m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O48">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="P48" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q48" t="str">
-        <v>Configured GitHub Actions CI pipeline (.github/workflows/ci.yml) to run tests on git push</v>
+        <v>Wrote comprehensive 77-case automated test suite covering Auth, Org, Projects, Tasks, and Attendance</v>
       </c>
     </row>
     <row r="49">
@@ -3347,13 +3347,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>2026-10-20</v>
+        <v>2026-10-19</v>
       </c>
       <c r="C49" t="str">
         <v>October 2026</v>
       </c>
       <c r="D49" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="E49" t="str">
         <v>ST-ENG-102</v>
@@ -3377,22 +3377,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L49" t="str">
-        <v>08:59 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M49" t="str">
-        <v>05:05 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N49" t="str">
-        <v>8h 6m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O49">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="P49" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q49" t="str">
-        <v>Wrote comprehensive 77-case automated test suite covering Auth, Org, Projects, Tasks, and Attendance</v>
+        <v>Added Export Excel (3 Months) direct download button in attendance portal header</v>
       </c>
     </row>
     <row r="50">
@@ -3400,13 +3400,13 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-16</v>
       </c>
       <c r="C50" t="str">
         <v>October 2026</v>
       </c>
       <c r="D50" t="str">
-        <v>Monday</v>
+        <v>Friday</v>
       </c>
       <c r="E50" t="str">
         <v>ST-ENG-102</v>
@@ -3445,7 +3445,7 @@
         <v>PRESENT</v>
       </c>
       <c r="Q50" t="str">
-        <v>Added Export Excel (3 Months) direct download button in attendance portal header</v>
+        <v>Added auto-fitting column widths and monthly aggregation formulas to generated Excel report</v>
       </c>
     </row>
     <row r="51">
@@ -3453,13 +3453,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>2026-10-16</v>
+        <v>2026-10-15</v>
       </c>
       <c r="C51" t="str">
         <v>October 2026</v>
       </c>
       <c r="D51" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="E51" t="str">
         <v>ST-ENG-102</v>
@@ -3483,22 +3483,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L51" t="str">
-        <v>09:06 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M51" t="str">
-        <v>05:08 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N51" t="str">
-        <v>8h 2m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O51">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="P51" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q51" t="str">
-        <v>Added auto-fitting column widths and monthly aggregation formulas to generated Excel report</v>
+        <v>Built generate-excel utility creating multi-sheet workbook for executive overview and attendance logs</v>
       </c>
     </row>
     <row r="52">
@@ -3506,13 +3506,13 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-14</v>
       </c>
       <c r="C52" t="str">
         <v>October 2026</v>
       </c>
       <c r="D52" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="E52" t="str">
         <v>ST-ENG-102</v>
@@ -3536,22 +3536,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L52" t="str">
-        <v>09:05 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M52" t="str">
-        <v>05:06 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N52" t="str">
-        <v>8h 1m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O52">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="P52" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q52" t="str">
-        <v>Built generate-excel utility creating multi-sheet workbook for executive overview and attendance logs</v>
+        <v>Researched Excel spreadsheet generation libraries in Node.js; evaluated SheetJS (xlsx)</v>
       </c>
     </row>
     <row r="53">
@@ -3559,13 +3559,13 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>2026-10-14</v>
+        <v>2026-10-13</v>
       </c>
       <c r="C53" t="str">
         <v>October 2026</v>
       </c>
       <c r="D53" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="E53" t="str">
         <v>ST-ENG-102</v>
@@ -3589,22 +3589,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L53" t="str">
-        <v>09:04 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M53" t="str">
-        <v>05:04 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N53" t="str">
-        <v>8h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O53">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="P53" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q53" t="str">
-        <v>Researched Excel spreadsheet generation libraries in Node.js; evaluated SheetJS (xlsx)</v>
+        <v>Added animated CSS pulse indicators and smooth hover elevation effects on engineering pod cards</v>
       </c>
     </row>
     <row r="54">
@@ -3612,13 +3612,13 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="C54" t="str">
         <v>October 2026</v>
       </c>
       <c r="D54" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="E54" t="str">
         <v>ST-ENG-102</v>
@@ -3642,22 +3642,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L54" t="str">
-        <v>09:03 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M54" t="str">
-        <v>05:14 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N54" t="str">
-        <v>8h 11m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O54">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="P54" t="str">
-        <v>REGULARIZED</v>
+        <v>PRESENT</v>
       </c>
       <c r="Q54" t="str">
-        <v>Added animated CSS pulse indicators and smooth hover elevation effects on engineering pod cards</v>
+        <v>Configured organizational hierarchy: Abhishek Kumar (VP &amp; Head) -&gt; Rohit Verma (Lead) -&gt; Nitesh Goel (SWE Intern)</v>
       </c>
     </row>
     <row r="55">
@@ -3665,13 +3665,13 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-09</v>
       </c>
       <c r="C55" t="str">
         <v>October 2026</v>
       </c>
       <c r="D55" t="str">
-        <v>Monday</v>
+        <v>Friday</v>
       </c>
       <c r="E55" t="str">
         <v>ST-ENG-102</v>
@@ -3695,22 +3695,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L55" t="str">
-        <v>09:02 AM</v>
+        <v>08:58 AM</v>
       </c>
       <c r="M55" t="str">
-        <v>05:12 PM</v>
+        <v>05:03 PM</v>
       </c>
       <c r="N55" t="str">
-        <v>8h 10m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O55">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="P55" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q55" t="str">
-        <v>Configured organizational hierarchy: Abhishek Kumar (VP &amp; Head) -&gt; Rohit Verma (Lead) -&gt; Nitesh Goel (SWE Intern)</v>
+        <v>Designed multi-tier Engineering Work Hierarchy matrix component in pages/portal/engineering/index.tsx</v>
       </c>
     </row>
     <row r="56">
@@ -3718,13 +3718,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-08</v>
       </c>
       <c r="C56" t="str">
         <v>October 2026</v>
       </c>
       <c r="D56" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="E56" t="str">
         <v>ST-ENG-102</v>
@@ -3748,22 +3748,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L56" t="str">
-        <v>08:59 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M56" t="str">
-        <v>05:06 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N56" t="str">
-        <v>8h 7m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O56">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="P56" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q56" t="str">
-        <v>Designed multi-tier Engineering Work Hierarchy matrix component in pages/portal/engineering/index.tsx</v>
+        <v>Updated attendance correction modal to submit timestamps with +05:30 IST offset</v>
       </c>
     </row>
     <row r="57">
@@ -3771,13 +3771,13 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-07</v>
       </c>
       <c r="C57" t="str">
         <v>October 2026</v>
       </c>
       <c r="D57" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="E57" t="str">
         <v>ST-ENG-102</v>
@@ -3801,22 +3801,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L57" t="str">
-        <v>08:58 AM</v>
+        <v>09:03 AM</v>
       </c>
       <c r="M57" t="str">
-        <v>05:04 PM</v>
+        <v>05:08 PM</v>
       </c>
       <c r="N57" t="str">
-        <v>8h 6m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O57">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="P57" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q57" t="str">
-        <v>Updated attendance correction modal to submit timestamps with +05:30 IST offset</v>
+        <v>Calibrated standard shift working hours to 09:00 AM - 05:00 PM (8-hour shift) across all portal modules</v>
       </c>
     </row>
     <row r="58">
@@ -3824,13 +3824,13 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-06</v>
       </c>
       <c r="C58" t="str">
         <v>October 2026</v>
       </c>
       <c r="D58" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="E58" t="str">
         <v>ST-ENG-102</v>
@@ -3854,10 +3854,10 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L58" t="str">
-        <v>09:08 AM</v>
+        <v>09:02 AM</v>
       </c>
       <c r="M58" t="str">
-        <v>05:13 PM</v>
+        <v>05:07 PM</v>
       </c>
       <c r="N58" t="str">
         <v>8h 5m</v>
@@ -3869,7 +3869,7 @@
         <v>PRESENT</v>
       </c>
       <c r="Q58" t="str">
-        <v>Calibrated standard shift working hours to 09:00 AM - 05:00 PM (8-hour shift) across all portal modules</v>
+        <v>Implemented formatAttendanceTime helper with explicit Asia/Kolkata timezone normalization</v>
       </c>
     </row>
     <row r="59">
@@ -3877,13 +3877,13 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C59" t="str">
         <v>October 2026</v>
       </c>
       <c r="D59" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="E59" t="str">
         <v>ST-ENG-102</v>
@@ -3907,22 +3907,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L59" t="str">
-        <v>09:07 AM</v>
+        <v>09:01 AM</v>
       </c>
       <c r="M59" t="str">
-        <v>05:11 PM</v>
+        <v>05:06 PM</v>
       </c>
       <c r="N59" t="str">
-        <v>8h 4m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O59">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P59" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q59" t="str">
-        <v>Implemented formatAttendanceTime helper with explicit Asia/Kolkata timezone normalization</v>
+        <v>Investigated timezone offset bug where UTC timestamps showed as afternoon check-ins on client devices</v>
       </c>
     </row>
     <row r="60">
@@ -3930,13 +3930,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C60" t="str">
         <v>October 2026</v>
       </c>
       <c r="D60" t="str">
-        <v>Monday</v>
+        <v>Friday</v>
       </c>
       <c r="E60" t="str">
         <v>ST-ENG-102</v>
@@ -3960,22 +3960,22 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L60" t="str">
-        <v>09:06 AM</v>
+        <v>08:58 AM</v>
       </c>
       <c r="M60" t="str">
-        <v>05:09 PM</v>
+        <v>05:03 PM</v>
       </c>
       <c r="N60" t="str">
-        <v>8h 3m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O60">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="P60" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q60" t="str">
-        <v>Investigated timezone offset bug where UTC timestamps showed as afternoon check-ins on client devices</v>
+        <v>System health monitoring, package dependency security audit, and edge caching review</v>
       </c>
     </row>
     <row r="61">
@@ -3983,13 +3983,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-01</v>
       </c>
       <c r="C61" t="str">
         <v>October 2026</v>
       </c>
       <c r="D61" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="E61" t="str">
         <v>ST-ENG-102</v>
@@ -4013,80 +4013,27 @@
         <v>09:00 AM – 05:00 PM (8 Hours)</v>
       </c>
       <c r="L61" t="str">
-        <v>09:03 AM</v>
+        <v>09:04 AM</v>
       </c>
       <c r="M61" t="str">
-        <v>05:03 PM</v>
+        <v>05:09 PM</v>
       </c>
       <c r="N61" t="str">
-        <v>8h 0m</v>
+        <v>8h 5m</v>
       </c>
       <c r="O61">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="P61" t="str">
         <v>PRESENT</v>
       </c>
       <c r="Q61" t="str">
-        <v>System health monitoring, package dependency security audit, and edge caching review</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62" t="str">
-        <v>2026-10-01</v>
-      </c>
-      <c r="C62" t="str">
-        <v>October 2026</v>
-      </c>
-      <c r="D62" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="E62" t="str">
-        <v>ST-ENG-102</v>
-      </c>
-      <c r="F62" t="str">
-        <v>Nitesh Goel</v>
-      </c>
-      <c r="G62" t="str">
-        <v>Engineering &amp; Technology</v>
-      </c>
-      <c r="H62" t="str">
-        <v>Software Engineering Trainee (SWE Trainee)</v>
-      </c>
-      <c r="I62" t="str">
-        <v>Abhishek Kumar (VP of Engineering &amp; Head of Technology)</v>
-      </c>
-      <c r="J62" t="str">
-        <v>Rohit Verma (Engineering Lead &amp; Principal PM)</v>
-      </c>
-      <c r="K62" t="str">
-        <v>09:00 AM – 05:00 PM (8 Hours)</v>
-      </c>
-      <c r="L62" t="str">
-        <v>09:02 AM</v>
-      </c>
-      <c r="M62" t="str">
-        <v>05:13 PM</v>
-      </c>
-      <c r="N62" t="str">
-        <v>8h 11m</v>
-      </c>
-      <c r="O62">
-        <v>491</v>
-      </c>
-      <c r="P62" t="str">
-        <v>PRESENT</v>
-      </c>
-      <c r="Q62" t="str">
         <v>October sprint kickoff; assigned to Timezone Calibration and Data Reporting deliverables</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q61"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>